<commit_message>
update replication section with latest work
</commit_message>
<xml_diff>
--- a/replication/delivered/tables/portfolio_backtest_summary.xlsx
+++ b/replication/delivered/tables/portfolio_backtest_summary.xlsx
@@ -8,24 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Pós-Graduação (Data Science for Finance NOVA IMS)\Asset Pricing &amp; Portfolio Management\10 assets, 5 year dataset with 3 year testing and 2 year rolling window\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED526EAE-DD9D-44C6-B031-DA90AC60A88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C64A08F-9439-4326-9A6E-45ABB6616D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1740" windowWidth="29040" windowHeight="15720" tabRatio="769" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1740" windowWidth="29040" windowHeight="15720" tabRatio="878" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Performance - No Rebalancing" sheetId="1" r:id="rId1"/>
-    <sheet name="Performance - Quarterly 0bps" sheetId="2" r:id="rId2"/>
-    <sheet name="Performance - Quarterly 10bps" sheetId="3" r:id="rId3"/>
-    <sheet name="Annual Returns - Fees" sheetId="4" r:id="rId4"/>
-    <sheet name="Cumulative Returns - Fees" sheetId="5" r:id="rId5"/>
-    <sheet name="Turnover" sheetId="6" r:id="rId6"/>
+    <sheet name="Mean Stats-No Rebalancing" sheetId="1" r:id="rId1"/>
+    <sheet name="Mean Stats-Quarterly 0bps" sheetId="2" r:id="rId2"/>
+    <sheet name="Mean Stats-Quarterly 15.0bps" sheetId="3" r:id="rId3"/>
+    <sheet name="Median Stats-No Rebalancing" sheetId="4" r:id="rId4"/>
+    <sheet name="Median Stats-Quarterly 0bps" sheetId="5" r:id="rId5"/>
+    <sheet name="Median Stats-Quarterly 15.0bps" sheetId="6" r:id="rId6"/>
+    <sheet name="SP500 Benchmark" sheetId="7" r:id="rId7"/>
+    <sheet name="Test Fees - Returns" sheetId="8" r:id="rId8"/>
+    <sheet name="Test Fees - Cumulative Returns" sheetId="9" r:id="rId9"/>
+    <sheet name="Turnover" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="46">
   <si>
     <t>Average Annual Return</t>
   </si>
@@ -99,6 +103,12 @@
     <t>Strategy</t>
   </si>
   <si>
+    <t>S&amp;P 500 ETF — Buy &amp; Hold (Mean)</t>
+  </si>
+  <si>
+    <t>S&amp;P 500 ETF — Buy &amp; Hold (Median)</t>
+  </si>
+  <si>
     <t>No Rebalancing</t>
   </si>
   <si>
@@ -147,7 +157,16 @@
     <t>Transaction Cost (50 bps)</t>
   </si>
   <si>
-    <t>Quarterly Rebalancing</t>
+    <t>No Rebalancing — Mean</t>
+  </si>
+  <si>
+    <t>No Rebalancing — Median</t>
+  </si>
+  <si>
+    <t>Quarterly Rebalancing — Mean</t>
+  </si>
+  <si>
+    <t>Quarterly Rebalancing — Median</t>
   </si>
 </sst>
 </file>
@@ -539,46 +558,46 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>0.131077172098511</v>
+        <v>0.13783290476702831</v>
       </c>
       <c r="C2">
-        <v>0.43493137445058588</v>
+        <v>0.46491044208419929</v>
       </c>
       <c r="D2">
-        <v>0.1545257895701439</v>
+        <v>0.15610412559370801</v>
       </c>
       <c r="E2">
-        <v>0.88635721644538534</v>
+        <v>0.92292394260422728</v>
       </c>
       <c r="F2">
-        <v>1.26378455481993</v>
+        <v>1.3249136399520289</v>
       </c>
       <c r="G2">
-        <v>0.75799932423466165</v>
+        <v>0.80809320351836544</v>
       </c>
       <c r="H2">
-        <v>3.970909842410264</v>
+        <v>4.0768522966590366</v>
       </c>
       <c r="I2">
-        <v>4.0071150803686881E-2</v>
+        <v>4.0250405845176473E-2</v>
       </c>
       <c r="J2">
-        <v>0.19635730406015461</v>
+        <v>0.19716995843191901</v>
       </c>
       <c r="K2">
-        <v>0.55106949250794879</v>
+        <v>0.55135099337748361</v>
       </c>
       <c r="L2">
-        <v>-0.33158717661547049</v>
+        <v>-0.27144461901408767</v>
       </c>
       <c r="M2">
-        <v>7.1423394139275276</v>
+        <v>8.0766780837092362</v>
       </c>
       <c r="N2">
-        <v>-1.5491202737696389E-2</v>
+        <v>-1.5627935201774579E-2</v>
       </c>
       <c r="O2">
-        <v>-1.9558731655632908E-2</v>
+        <v>-1.97370101130105E-2</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -586,46 +605,46 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <v>0.18941950575474251</v>
+        <v>0.1885128980164322</v>
       </c>
       <c r="C3">
-        <v>0.67502490657370995</v>
+        <v>0.66018348136032245</v>
       </c>
       <c r="D3">
-        <v>0.2337344033397569</v>
+        <v>0.23837975920546531</v>
       </c>
       <c r="E3">
-        <v>0.83994047842937969</v>
+        <v>0.8119314205735203</v>
       </c>
       <c r="F3">
-        <v>1.2343079329262849</v>
+        <v>1.1920748272607291</v>
       </c>
       <c r="G3">
-        <v>0.76663048499292497</v>
+        <v>0.72303523807653802</v>
       </c>
       <c r="H3">
-        <v>3.6798857114869059</v>
+        <v>3.4143411483971779</v>
       </c>
       <c r="I3">
-        <v>7.5792845633059797E-2</v>
+        <v>7.8501789505987032E-2</v>
       </c>
       <c r="J3">
-        <v>0.27829243670777543</v>
+        <v>0.28361435187078038</v>
       </c>
       <c r="K3">
-        <v>0.53918906669945732</v>
+        <v>0.53757615894039734</v>
       </c>
       <c r="L3">
-        <v>2.357243583822533E-3</v>
+        <v>-2.1318439339279349E-2</v>
       </c>
       <c r="M3">
-        <v>5.7161217373742099</v>
+        <v>6.8828679956810497</v>
       </c>
       <c r="N3">
-        <v>-2.3466968357938409E-2</v>
+        <v>-2.395189938246672E-2</v>
       </c>
       <c r="O3">
-        <v>-2.9619478222769349E-2</v>
+        <v>-3.0226687343209269E-2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -633,46 +652,46 @@
         <v>16</v>
       </c>
       <c r="B4">
-        <v>8.6045306736299759E-2</v>
+        <v>9.5474406826550395E-2</v>
       </c>
       <c r="C4">
-        <v>0.27348499770369988</v>
+        <v>0.31491622066129399</v>
       </c>
       <c r="D4">
-        <v>0.1211720427419655</v>
+        <v>0.1202020578723792</v>
       </c>
       <c r="E4">
-        <v>0.75131838452317945</v>
+        <v>0.82911208815342985</v>
       </c>
       <c r="F4">
-        <v>1.0646785860418</v>
+        <v>1.1824860598950411</v>
       </c>
       <c r="G4">
-        <v>0.58828996410253886</v>
+        <v>0.68760908984251601</v>
       </c>
       <c r="H4">
-        <v>2.7319961671735542</v>
+        <v>2.9905169039175821</v>
       </c>
       <c r="I4">
-        <v>4.6362591257585163E-2</v>
+        <v>4.199110501466511E-2</v>
       </c>
       <c r="J4">
-        <v>0.17425471838712461</v>
+        <v>0.16638915675451679</v>
       </c>
       <c r="K4">
-        <v>0.54061814253341989</v>
+        <v>0.54471523178807957</v>
       </c>
       <c r="L4">
-        <v>-0.46463101091298847</v>
+        <v>-0.48385273498022652</v>
       </c>
       <c r="M4">
-        <v>6.2687468735431704</v>
+        <v>6.3869973617371114</v>
       </c>
       <c r="N4">
-        <v>-1.221391748237206E-2</v>
+        <v>-1.207599442839883E-2</v>
       </c>
       <c r="O4">
-        <v>-1.5403487257549661E-2</v>
+        <v>-1.524003162731211E-2</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -680,46 +699,46 @@
         <v>17</v>
       </c>
       <c r="B5">
-        <v>0.19986373794438819</v>
+        <v>0.2205461961043246</v>
       </c>
       <c r="C5">
-        <v>0.70509485683100503</v>
+        <v>0.80540501844658929</v>
       </c>
       <c r="D5">
-        <v>0.26713082293630919</v>
+        <v>0.27019003803776898</v>
       </c>
       <c r="E5">
-        <v>0.79064530395339394</v>
+        <v>0.83280077673533259</v>
       </c>
       <c r="F5">
-        <v>1.1730853666845971</v>
+        <v>1.2329977291597589</v>
       </c>
       <c r="G5">
-        <v>0.72902182770447566</v>
+        <v>0.79948954330844979</v>
       </c>
       <c r="H5">
-        <v>3.3968843853804058</v>
+        <v>3.5133600250492441</v>
       </c>
       <c r="I5">
-        <v>9.3286265080366096E-2</v>
+        <v>8.902545767804515E-2</v>
       </c>
       <c r="J5">
-        <v>0.31324020177250811</v>
+        <v>0.29839213165119233</v>
       </c>
       <c r="K5">
-        <v>0.53081788957788045</v>
+        <v>0.53141721854304647</v>
       </c>
       <c r="L5">
-        <v>7.9744266287177512E-2</v>
+        <v>2.4493888010669571E-2</v>
       </c>
       <c r="M5">
-        <v>5.4700637363673863</v>
+        <v>6.0524668718376917</v>
       </c>
       <c r="N5">
-        <v>-2.6885927709086401E-2</v>
+        <v>-2.7120838213829091E-2</v>
       </c>
       <c r="O5">
-        <v>-3.3917519977200279E-2</v>
+        <v>-3.4232957143065318E-2</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -727,46 +746,46 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>0.13434919632155981</v>
+        <v>0.13287575745591079</v>
       </c>
       <c r="C6">
-        <v>0.46772470388705267</v>
+        <v>0.4565947781552081</v>
       </c>
       <c r="D6">
-        <v>0.16422266958311099</v>
+        <v>0.16664298382965559</v>
       </c>
       <c r="E6">
-        <v>0.80480702824924066</v>
+        <v>0.80057999531152158</v>
       </c>
       <c r="F6">
-        <v>1.166969485319844</v>
+        <v>1.1651048624916081</v>
       </c>
       <c r="G6">
-        <v>0.7228223765657692</v>
+        <v>0.67531750244167355</v>
       </c>
       <c r="H6">
-        <v>3.549710287851783</v>
+        <v>3.3371326375764698</v>
       </c>
       <c r="I6">
-        <v>5.7172438474761798E-2</v>
+        <v>5.9365322801388648E-2</v>
       </c>
       <c r="J6">
-        <v>0.20841951243760479</v>
+        <v>0.21814714053885439</v>
       </c>
       <c r="K6">
-        <v>0.54031319057740623</v>
+        <v>0.53645033112582785</v>
       </c>
       <c r="L6">
-        <v>-0.17083458431121221</v>
+        <v>-0.13340146098305011</v>
       </c>
       <c r="M6">
-        <v>5.3288752853395911</v>
+        <v>6.0099851787588072</v>
       </c>
       <c r="N6">
-        <v>-1.6482970812656469E-2</v>
+        <v>-1.6739601167760479E-2</v>
       </c>
       <c r="O6">
-        <v>-2.0805747349622958E-2</v>
+        <v>-2.1126086799601668E-2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -774,46 +793,46 @@
         <v>19</v>
       </c>
       <c r="B7">
-        <v>0.12102960693777599</v>
+        <v>0.12671256433829681</v>
       </c>
       <c r="C7">
-        <v>0.39823276722133849</v>
+        <v>0.42402195275474908</v>
       </c>
       <c r="D7">
-        <v>0.14386411622022471</v>
+        <v>0.14350318464325529</v>
       </c>
       <c r="E7">
-        <v>0.87745624052072513</v>
+        <v>0.92271310653672745</v>
       </c>
       <c r="F7">
-        <v>1.248714333272795</v>
+        <v>1.3220826827737071</v>
       </c>
       <c r="G7">
-        <v>0.74330521428781626</v>
+        <v>0.80605515995283095</v>
       </c>
       <c r="H7">
-        <v>3.8924100781133508</v>
+        <v>4.0178238381636469</v>
       </c>
       <c r="I7">
-        <v>3.7821593045040257E-2</v>
+        <v>3.7366233751437029E-2</v>
       </c>
       <c r="J7">
-        <v>0.18654236844863659</v>
+        <v>0.1836695914817652</v>
       </c>
       <c r="K7">
-        <v>0.55101624888014467</v>
+        <v>0.55202649006622528</v>
       </c>
       <c r="L7">
-        <v>-0.36716500719279832</v>
+        <v>-0.32093811900597308</v>
       </c>
       <c r="M7">
-        <v>7.1275572193895762</v>
+        <v>7.8483652241164341</v>
       </c>
       <c r="N7">
-        <v>-1.4426353665874459E-2</v>
+        <v>-1.4366403947245509E-2</v>
       </c>
       <c r="O7">
-        <v>-1.821323904343481E-2</v>
+        <v>-1.8143788647729201E-2</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -821,46 +840,46 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>0.10986625441198231</v>
+        <v>0.1171359949159449</v>
       </c>
       <c r="C8">
-        <v>0.36240436332752851</v>
+        <v>0.39377931754804829</v>
       </c>
       <c r="D8">
-        <v>0.13061106513761719</v>
+        <v>0.13070302031217379</v>
       </c>
       <c r="E8">
-        <v>0.87212122335985331</v>
+        <v>0.93081540219204062</v>
       </c>
       <c r="F8">
-        <v>1.2405766171257491</v>
+        <v>1.3311291363965461</v>
       </c>
       <c r="G8">
-        <v>0.73797781743398305</v>
+        <v>0.80838527839371221</v>
       </c>
       <c r="H8">
-        <v>3.8819840565493342</v>
+        <v>4.0612268095190789</v>
       </c>
       <c r="I8">
-        <v>3.871187514593382E-2</v>
+        <v>3.6623790907133927E-2</v>
       </c>
       <c r="J8">
-        <v>0.1739597895055266</v>
+        <v>0.16938668885836819</v>
       </c>
       <c r="K8">
-        <v>0.55081778417973892</v>
+        <v>0.55202649006622517</v>
       </c>
       <c r="L8">
-        <v>-0.39560895716607941</v>
+        <v>-0.38289075319775112</v>
       </c>
       <c r="M8">
-        <v>6.7733996828851346</v>
+        <v>7.4870470415014996</v>
       </c>
       <c r="N8">
-        <v>-1.309742402535331E-2</v>
+        <v>-1.30781038797078E-2</v>
       </c>
       <c r="O8">
-        <v>-1.653545392267728E-2</v>
+        <v>-1.651855428129002E-2</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -868,46 +887,46 @@
         <v>21</v>
       </c>
       <c r="B9">
-        <v>0.1046243249782412</v>
+        <v>0.112590074344571</v>
       </c>
       <c r="C9">
-        <v>0.34701722256327477</v>
+        <v>0.38201090215017092</v>
       </c>
       <c r="D9">
-        <v>0.12666745589630801</v>
+        <v>0.12738680749486619</v>
       </c>
       <c r="E9">
-        <v>0.86757109919762398</v>
+        <v>0.91777893113177711</v>
       </c>
       <c r="F9">
-        <v>1.2413084718613721</v>
+        <v>1.3175766879431821</v>
       </c>
       <c r="G9">
-        <v>0.73997424741945661</v>
+        <v>0.79508796973535212</v>
       </c>
       <c r="H9">
-        <v>3.7241583341482292</v>
+        <v>3.8781679939496838</v>
       </c>
       <c r="I9">
-        <v>4.2909570808663533E-2</v>
+        <v>3.966168416740655E-2</v>
       </c>
       <c r="J9">
-        <v>0.17114132938086121</v>
+        <v>0.1663149807402732</v>
       </c>
       <c r="K9">
-        <v>0.54788982380944018</v>
+        <v>0.54962913907284761</v>
       </c>
       <c r="L9">
-        <v>-0.39533855301923271</v>
+        <v>-0.40841409705673842</v>
       </c>
       <c r="M9">
-        <v>6.2772497733624224</v>
+        <v>6.9760252177348194</v>
       </c>
       <c r="N9">
-        <v>-1.270960416349249E-2</v>
+        <v>-1.275253041028488E-2</v>
       </c>
       <c r="O9">
-        <v>-1.6043827798608142E-2</v>
+        <v>-1.6105689288750131E-2</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -915,46 +934,226 @@
         <v>22</v>
       </c>
       <c r="B10">
-        <v>0.118115864066305</v>
+        <v>0.1263792223054313</v>
       </c>
       <c r="C10">
-        <v>0.39510725866186708</v>
+        <v>0.43198005984657639</v>
       </c>
       <c r="D10">
-        <v>0.13922794069696851</v>
+        <v>0.14166887210846149</v>
       </c>
       <c r="E10">
-        <v>0.87926251803479372</v>
+        <v>0.92212077078482424</v>
       </c>
       <c r="F10">
-        <v>1.2598395788433789</v>
+        <v>1.3280873565560589</v>
       </c>
       <c r="G10">
-        <v>0.75199786729315321</v>
+        <v>0.8019479017483363</v>
       </c>
       <c r="H10">
-        <v>3.7477975474350091</v>
+        <v>3.9312036682962281</v>
       </c>
       <c r="I10">
-        <v>4.3547430708480203E-2</v>
+        <v>4.1744896361555588E-2</v>
       </c>
       <c r="J10">
-        <v>0.18135071139938649</v>
+        <v>0.17999444347052129</v>
       </c>
       <c r="K10">
-        <v>0.55008950058847306</v>
+        <v>0.54992052980132455</v>
       </c>
       <c r="L10">
-        <v>-0.33549715195574392</v>
+        <v>-0.31306022539286138</v>
       </c>
       <c r="M10">
-        <v>6.1602436259717184</v>
+        <v>7.2479384399552176</v>
       </c>
       <c r="N10">
-        <v>-1.3957533993535529E-2</v>
+        <v>-1.4177662533858781E-2</v>
       </c>
       <c r="O10">
-        <v>-1.7622382926163721E-2</v>
+        <v>-1.7906763259864421E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>2.4</v>
+      </c>
+      <c r="E2">
+        <v>2.44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>2.19</v>
+      </c>
+      <c r="E3">
+        <v>2.12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1.89</v>
+      </c>
+      <c r="E4">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="E5">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E6">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0.54</v>
+      </c>
+      <c r="E7">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0.27</v>
+      </c>
+      <c r="E8">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0.26</v>
+      </c>
+      <c r="E9">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0.26</v>
+      </c>
+      <c r="E10">
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -1016,46 +1215,46 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>0.13153948434986731</v>
+        <v>0.1384385468620204</v>
       </c>
       <c r="C2">
-        <v>0.43808458186343813</v>
+        <v>0.46840506695585937</v>
       </c>
       <c r="D2">
-        <v>0.15229696577139351</v>
+        <v>0.15346903892985511</v>
       </c>
       <c r="E2">
-        <v>0.908862639261236</v>
+        <v>0.9495608666656874</v>
       </c>
       <c r="F2">
-        <v>1.2980598982889591</v>
+        <v>1.3671085532439911</v>
       </c>
       <c r="G2">
-        <v>0.76824131191256095</v>
+        <v>0.83854249530671154</v>
       </c>
       <c r="H2">
-        <v>4.0262362399934091</v>
+        <v>4.1652590609489559</v>
       </c>
       <c r="I2">
-        <v>4.0090623267911969E-2</v>
+        <v>3.9745734706193157E-2</v>
       </c>
       <c r="J2">
-        <v>0.1960691591994933</v>
+        <v>0.19493806560492091</v>
       </c>
       <c r="K2">
-        <v>0.55154641909814328</v>
+        <v>0.55047682119205299</v>
       </c>
       <c r="L2">
-        <v>-0.3352005033952184</v>
+        <v>-0.27579465628299588</v>
       </c>
       <c r="M2">
-        <v>7.0016146928209206</v>
+        <v>7.624257850341281</v>
       </c>
       <c r="N2">
-        <v>-1.5258426271507929E-2</v>
+        <v>-1.5352494617471121E-2</v>
       </c>
       <c r="O2">
-        <v>-1.9267286631402321E-2</v>
+        <v>-1.939220705376803E-2</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1063,46 +1262,46 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <v>0.16527151482840949</v>
+        <v>0.17439981214070591</v>
       </c>
       <c r="C3">
-        <v>0.56655798033003846</v>
+        <v>0.62118047762755524</v>
       </c>
       <c r="D3">
-        <v>0.22810678071351631</v>
+        <v>0.23102131880941931</v>
       </c>
       <c r="E3">
-        <v>0.73328898046241453</v>
+        <v>0.75600613681250872</v>
       </c>
       <c r="F3">
-        <v>1.0653836083994821</v>
+        <v>1.105990397096581</v>
       </c>
       <c r="G3">
-        <v>0.65069326073613842</v>
+        <v>0.67347393765305352</v>
       </c>
       <c r="H3">
-        <v>2.917044154964163</v>
+        <v>3.1142599712880372</v>
       </c>
       <c r="I3">
-        <v>7.4961597532454738E-2</v>
+        <v>7.6117340066545552E-2</v>
       </c>
       <c r="J3">
-        <v>0.25778570919310467</v>
+        <v>0.26001798881136112</v>
       </c>
       <c r="K3">
-        <v>0.53841472412036462</v>
+        <v>0.53950362745270264</v>
       </c>
       <c r="L3">
-        <v>-9.057421240008813E-2</v>
+        <v>1.3555955052952789E-2</v>
       </c>
       <c r="M3">
-        <v>5.2654212038986987</v>
+        <v>6.7795896109448064</v>
       </c>
       <c r="N3">
-        <v>-2.2979681752969199E-2</v>
+        <v>-2.324545124408826E-2</v>
       </c>
       <c r="O3">
-        <v>-2.89840576536564E-2</v>
+        <v>-2.9326545523115342E-2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1110,46 +1309,46 @@
         <v>16</v>
       </c>
       <c r="B4">
-        <v>8.4738548852253043E-2</v>
+        <v>9.1128043600765304E-2</v>
       </c>
       <c r="C4">
-        <v>0.26924640435365571</v>
+        <v>0.29728144689183128</v>
       </c>
       <c r="D4">
-        <v>0.11671171436509151</v>
+        <v>0.11667080708957191</v>
       </c>
       <c r="E4">
-        <v>0.7775375374602137</v>
+        <v>0.82879778861885056</v>
       </c>
       <c r="F4">
-        <v>1.1041104684020211</v>
+        <v>1.183471815228329</v>
       </c>
       <c r="G4">
-        <v>0.61052286771010533</v>
+        <v>0.68131420732115155</v>
       </c>
       <c r="H4">
-        <v>2.6004380655404158</v>
+        <v>2.8031312920805651</v>
       </c>
       <c r="I4">
-        <v>4.4940086735702739E-2</v>
+        <v>4.2531704567217957E-2</v>
       </c>
       <c r="J4">
-        <v>0.1683791330480077</v>
+        <v>0.16282741817619781</v>
       </c>
       <c r="K4">
-        <v>0.5395585574507703</v>
+        <v>0.54343046357615887</v>
       </c>
       <c r="L4">
-        <v>-0.49896144116272201</v>
+        <v>-0.48891231095109472</v>
       </c>
       <c r="M4">
-        <v>6.4339501504339687</v>
+        <v>6.3606757879055804</v>
       </c>
       <c r="N4">
-        <v>-1.175694147026588E-2</v>
+        <v>-1.172734768251737E-2</v>
       </c>
       <c r="O4">
-        <v>-1.4829103564130889E-2</v>
+        <v>-1.4798432988316179E-2</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1157,46 +1356,46 @@
         <v>17</v>
       </c>
       <c r="B5">
-        <v>0.18303007458380149</v>
+        <v>0.18590777654257931</v>
       </c>
       <c r="C5">
-        <v>0.63559160557845107</v>
+        <v>0.64925650917638356</v>
       </c>
       <c r="D5">
-        <v>0.2621309101937741</v>
+        <v>0.26733153945072952</v>
       </c>
       <c r="E5">
-        <v>0.69622799088933462</v>
+        <v>0.69180129626983144</v>
       </c>
       <c r="F5">
-        <v>1.021367799053678</v>
+        <v>1.014938872086004</v>
       </c>
       <c r="G5">
-        <v>0.63986287036669964</v>
+        <v>0.64346157255128078</v>
       </c>
       <c r="H5">
-        <v>2.7689547827137408</v>
+        <v>2.788794690591136</v>
       </c>
       <c r="I5">
-        <v>9.2415300238401471E-2</v>
+        <v>9.5583797897072054E-2</v>
       </c>
       <c r="J5">
-        <v>0.28821336163639272</v>
+        <v>0.29612709227961359</v>
       </c>
       <c r="K5">
-        <v>0.53256795626821618</v>
+        <v>0.533133434047113</v>
       </c>
       <c r="L5">
-        <v>-3.7988855451693671E-2</v>
+        <v>1.494452841034E-2</v>
       </c>
       <c r="M5">
-        <v>5.555346071678847</v>
+        <v>7.8756425880218277</v>
       </c>
       <c r="N5">
-        <v>-2.643465680655015E-2</v>
+        <v>-2.6962105958495668E-2</v>
       </c>
       <c r="O5">
-        <v>-3.3334638100703022E-2</v>
+        <v>-3.3998981618003209E-2</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1204,46 +1403,46 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>0.10158371692667011</v>
+        <v>0.11622148753195</v>
       </c>
       <c r="C6">
-        <v>0.31900229526927992</v>
+        <v>0.38591447538770057</v>
       </c>
       <c r="D6">
-        <v>0.15895527140252599</v>
+        <v>0.16018540122519881</v>
       </c>
       <c r="E6">
-        <v>0.65273548381881308</v>
+        <v>0.73613415966449591</v>
       </c>
       <c r="F6">
-        <v>0.9319927393117402</v>
+        <v>1.057253458453554</v>
       </c>
       <c r="G6">
-        <v>0.5551345724382879</v>
+        <v>0.64309157352229784</v>
       </c>
       <c r="H6">
-        <v>2.4301004381793359</v>
+        <v>2.7882061463302859</v>
       </c>
       <c r="I6">
-        <v>5.5710760276600838E-2</v>
+        <v>5.5785524532996809E-2</v>
       </c>
       <c r="J6">
-        <v>0.1940160839737903</v>
+        <v>0.19302172783757751</v>
       </c>
       <c r="K6">
-        <v>0.53876397842851365</v>
+        <v>0.54052980132450335</v>
       </c>
       <c r="L6">
-        <v>-0.23136250501151201</v>
+        <v>-0.2184127724855395</v>
       </c>
       <c r="M6">
-        <v>4.430030636605764</v>
+        <v>4.8937750901732668</v>
       </c>
       <c r="N6">
-        <v>-1.60672056207261E-2</v>
+        <v>-1.613658040917549E-2</v>
       </c>
       <c r="O6">
-        <v>-2.0251330257052461E-2</v>
+        <v>-2.0353085327398199E-2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1251,46 +1450,46 @@
         <v>19</v>
       </c>
       <c r="B7">
-        <v>0.1205097591770521</v>
+        <v>0.1255307100957794</v>
       </c>
       <c r="C7">
-        <v>0.3982975934081035</v>
+        <v>0.42002647709978969</v>
       </c>
       <c r="D7">
-        <v>0.13993488862417719</v>
+        <v>0.13980234840588859</v>
       </c>
       <c r="E7">
-        <v>0.90547553529829206</v>
+        <v>0.94490790210247644</v>
       </c>
       <c r="F7">
-        <v>1.290464015529182</v>
+        <v>1.3560329854136099</v>
       </c>
       <c r="G7">
-        <v>0.7662928696355199</v>
+        <v>0.82145263293008086</v>
       </c>
       <c r="H7">
-        <v>3.9839836246694431</v>
+        <v>4.0637579567391802</v>
       </c>
       <c r="I7">
-        <v>3.7304474941513267E-2</v>
+        <v>3.679218773192687E-2</v>
       </c>
       <c r="J7">
-        <v>0.1834006815236234</v>
+        <v>0.1810183431353555</v>
       </c>
       <c r="K7">
-        <v>0.55170528923006668</v>
+        <v>0.55178807947019859</v>
       </c>
       <c r="L7">
-        <v>-0.38432747160100528</v>
+        <v>-0.3350713520432213</v>
       </c>
       <c r="M7">
-        <v>7.0446649082808381</v>
+        <v>7.6230213299713796</v>
       </c>
       <c r="N7">
-        <v>-1.402128555379329E-2</v>
+        <v>-1.3987627852952021E-2</v>
       </c>
       <c r="O7">
-        <v>-1.7704743232219811E-2</v>
+        <v>-1.7667596721049991E-2</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1298,46 +1497,46 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>0.1084888988507679</v>
+        <v>0.114238810862214</v>
       </c>
       <c r="C8">
-        <v>0.35820709601322298</v>
+        <v>0.38322856077875211</v>
       </c>
       <c r="D8">
-        <v>0.1254151123362329</v>
+        <v>0.12609569636639301</v>
       </c>
       <c r="E8">
-        <v>0.90797432787539323</v>
+        <v>0.94556703670374465</v>
       </c>
       <c r="F8">
-        <v>1.2932920842269899</v>
+        <v>1.352839512449421</v>
       </c>
       <c r="G8">
-        <v>0.75903484296371204</v>
+        <v>0.80313953372015812</v>
       </c>
       <c r="H8">
-        <v>3.8889560649986121</v>
+        <v>3.9808709213055948</v>
       </c>
       <c r="I8">
-        <v>3.76025840750914E-2</v>
+        <v>3.6158496854937799E-2</v>
       </c>
       <c r="J8">
-        <v>0.16943935240289729</v>
+        <v>0.166429646163889</v>
       </c>
       <c r="K8">
-        <v>0.5504997804205386</v>
+        <v>0.55068874172185434</v>
       </c>
       <c r="L8">
-        <v>-0.43630260524695907</v>
+        <v>-0.41902689469282178</v>
       </c>
       <c r="M8">
-        <v>6.6469802378700011</v>
+        <v>7.2081924743573476</v>
       </c>
       <c r="N8">
-        <v>-1.2564505673664961E-2</v>
+        <v>-1.2612207983952951E-2</v>
       </c>
       <c r="O8">
-        <v>-1.5865764302356991E-2</v>
+        <v>-1.5931381390698919E-2</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1345,46 +1544,46 @@
         <v>21</v>
       </c>
       <c r="B9">
-        <v>0.10205445913365251</v>
+        <v>0.1070717091014157</v>
       </c>
       <c r="C9">
-        <v>0.33579881525509653</v>
+        <v>0.3590485092877107</v>
       </c>
       <c r="D9">
-        <v>0.1215827913593638</v>
+        <v>0.12263033783536791</v>
       </c>
       <c r="E9">
-        <v>0.88693704713129562</v>
+        <v>0.91219538290485558</v>
       </c>
       <c r="F9">
-        <v>1.270621150952097</v>
+        <v>1.3078012335062921</v>
       </c>
       <c r="G9">
-        <v>0.71249261954746257</v>
+        <v>0.75151103248303597</v>
       </c>
       <c r="H9">
-        <v>3.3798169242262048</v>
+        <v>3.490700448210132</v>
       </c>
       <c r="I9">
-        <v>4.2460502154648049E-2</v>
+        <v>4.1092763736848177E-2</v>
       </c>
       <c r="J9">
-        <v>0.16857119552543429</v>
+        <v>0.16700775826279149</v>
       </c>
       <c r="K9">
-        <v>0.54534744497338705</v>
+        <v>0.54747019867549673</v>
       </c>
       <c r="L9">
-        <v>-0.41994432942653992</v>
+        <v>-0.438854440193991</v>
       </c>
       <c r="M9">
-        <v>6.0941689403280073</v>
+        <v>6.5735584312286992</v>
       </c>
       <c r="N9">
-        <v>-1.219294924462213E-2</v>
+        <v>-1.2281582139090089E-2</v>
       </c>
       <c r="O9">
-        <v>-1.539333101360295E-2</v>
+        <v>-1.550953811167719E-2</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1392,46 +1591,46 @@
         <v>22</v>
       </c>
       <c r="B10">
-        <v>0.1148532238115265</v>
+        <v>0.1218246221965317</v>
       </c>
       <c r="C10">
-        <v>0.38105005421365828</v>
+        <v>0.41357990961818719</v>
       </c>
       <c r="D10">
-        <v>0.1343622237142858</v>
+        <v>0.1372511838153247</v>
       </c>
       <c r="E10">
-        <v>0.89466801907360383</v>
+        <v>0.92202959970857246</v>
       </c>
       <c r="F10">
-        <v>1.283315664322257</v>
+        <v>1.328194231188633</v>
       </c>
       <c r="G10">
-        <v>0.72710573735128348</v>
+        <v>0.77996512412830099</v>
       </c>
       <c r="H10">
-        <v>3.4982850496347271</v>
+        <v>3.7052163029797591</v>
       </c>
       <c r="I10">
-        <v>4.3189257259873E-2</v>
+        <v>4.2825209732598603E-2</v>
       </c>
       <c r="J10">
-        <v>0.18038937196222471</v>
+        <v>0.17992423860390541</v>
       </c>
       <c r="K10">
-        <v>0.54680457427934026</v>
+        <v>0.54712582781456942</v>
       </c>
       <c r="L10">
-        <v>-0.36888476719427099</v>
+        <v>-0.35276079513470998</v>
       </c>
       <c r="M10">
-        <v>6.0123161392753843</v>
+        <v>6.8754407648286211</v>
       </c>
       <c r="N10">
-        <v>-1.346631465779936E-2</v>
+        <v>-1.373799298113115E-2</v>
       </c>
       <c r="O10">
-        <v>-1.7003085005043109E-2</v>
+        <v>-1.735080842600184E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1493,46 +1692,46 @@
         <v>14</v>
       </c>
       <c r="B2">
-        <v>0.13066606156267749</v>
+        <v>0.1375545697718549</v>
       </c>
       <c r="C2">
-        <v>0.4343256384880686</v>
+        <v>0.46451358760888461</v>
       </c>
       <c r="D2">
-        <v>0.15229663218855771</v>
+        <v>0.1534700198910198</v>
       </c>
       <c r="E2">
-        <v>0.90278367523619718</v>
+        <v>0.94351143864070042</v>
       </c>
       <c r="F2">
-        <v>1.2890889232406031</v>
+        <v>1.3580715865032369</v>
       </c>
       <c r="G2">
-        <v>0.76151447089521018</v>
+        <v>0.83205482818219179</v>
       </c>
       <c r="H2">
-        <v>3.9949945966891311</v>
+        <v>4.133629521438503</v>
       </c>
       <c r="I2">
-        <v>4.0168508901886987E-2</v>
+        <v>3.9818465071669543E-2</v>
       </c>
       <c r="J2">
-        <v>0.19617852016456391</v>
+        <v>0.19504572575826901</v>
       </c>
       <c r="K2">
-        <v>0.5512417657701969</v>
+        <v>0.55031788079470201</v>
       </c>
       <c r="L2">
-        <v>-0.33501089272535828</v>
+        <v>-0.27558616021905408</v>
       </c>
       <c r="M2">
-        <v>7.0005360902786462</v>
+        <v>7.6237425729463659</v>
       </c>
       <c r="N2">
-        <v>-1.526185767041701E-2</v>
+        <v>-1.5356104106377361E-2</v>
       </c>
       <c r="O2">
-        <v>-1.9270709249525779E-2</v>
+        <v>-1.9395842364175759E-2</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -1540,46 +1739,46 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <v>0.16166434417649281</v>
+        <v>0.17060223268595401</v>
       </c>
       <c r="C3">
-        <v>0.55046692084529936</v>
+        <v>0.60356291656536043</v>
       </c>
       <c r="D3">
-        <v>0.2281011840350394</v>
+        <v>0.2310480888276471</v>
       </c>
       <c r="E3">
-        <v>0.7165590166940734</v>
+        <v>0.73865236981426308</v>
       </c>
       <c r="F3">
-        <v>1.0407408276628261</v>
+        <v>1.0802402340814841</v>
       </c>
       <c r="G3">
-        <v>0.63123198769370559</v>
+        <v>0.65311742968260522</v>
       </c>
       <c r="H3">
-        <v>2.8348918693810998</v>
+        <v>3.0281879665488831</v>
       </c>
       <c r="I3">
-        <v>7.6009824000137061E-2</v>
+        <v>7.7352409289865739E-2</v>
       </c>
       <c r="J3">
-        <v>0.25889562330178362</v>
+        <v>0.26123698668084089</v>
       </c>
       <c r="K3">
-        <v>0.53779210216593176</v>
+        <v>0.53896058109508682</v>
       </c>
       <c r="L3">
-        <v>-9.0179357114679823E-2</v>
+        <v>1.3886832646332579E-2</v>
       </c>
       <c r="M3">
-        <v>5.2651159932101654</v>
+        <v>6.7787872081889358</v>
       </c>
       <c r="N3">
-        <v>-2.299341601656725E-2</v>
+        <v>-2.3263294807083348E-2</v>
       </c>
       <c r="O3">
-        <v>-2.899764459782244E-2</v>
+        <v>-2.934509374404215E-2</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1587,46 +1786,46 @@
         <v>16</v>
       </c>
       <c r="B4">
-        <v>8.3358962951623747E-2</v>
+        <v>8.9749457596787666E-2</v>
       </c>
       <c r="C4">
-        <v>0.26399359295411567</v>
+        <v>0.29193713447659531</v>
       </c>
       <c r="D4">
-        <v>0.11670822933216431</v>
+        <v>0.1166766662013677</v>
       </c>
       <c r="E4">
-        <v>0.76496417555905194</v>
+        <v>0.81644095682018814</v>
       </c>
       <c r="F4">
-        <v>1.0857502260313829</v>
+        <v>1.165332088602669</v>
       </c>
       <c r="G4">
-        <v>0.59815780875192859</v>
+        <v>0.66927364881377682</v>
       </c>
       <c r="H4">
-        <v>2.546837034495554</v>
+        <v>2.749531039265102</v>
       </c>
       <c r="I4">
-        <v>4.5232844126420403E-2</v>
+        <v>4.2809096203547357E-2</v>
       </c>
       <c r="J4">
-        <v>0.16880331732199391</v>
+        <v>0.16317348173638629</v>
       </c>
       <c r="K4">
-        <v>0.5390420011593795</v>
+        <v>0.54304635761589404</v>
       </c>
       <c r="L4">
-        <v>-0.4992702187383059</v>
+        <v>-0.48876611093641159</v>
       </c>
       <c r="M4">
-        <v>6.4306450900720167</v>
+        <v>6.3610201809108764</v>
       </c>
       <c r="N4">
-        <v>-1.176205491218273E-2</v>
+        <v>-1.1733425359854849E-2</v>
       </c>
       <c r="O4">
-        <v>-1.483412527073126E-2</v>
+        <v>-1.4804664893027151E-2</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -1634,46 +1833,46 @@
         <v>17</v>
       </c>
       <c r="B5">
-        <v>0.17896999876708239</v>
+        <v>0.18179980080629851</v>
       </c>
       <c r="C5">
-        <v>0.61725620077977095</v>
+        <v>0.63072737347659946</v>
       </c>
       <c r="D5">
-        <v>0.26214802398341652</v>
+        <v>0.26735031320538299</v>
       </c>
       <c r="E5">
-        <v>0.67970483883346444</v>
+        <v>0.67556620496234332</v>
       </c>
       <c r="F5">
-        <v>0.99703299315189609</v>
+        <v>0.9909993270645594</v>
       </c>
       <c r="G5">
-        <v>0.62044960362016677</v>
+        <v>0.6249903004194195</v>
       </c>
       <c r="H5">
-        <v>2.6916819029105641</v>
+        <v>2.7139273351906059</v>
       </c>
       <c r="I5">
-        <v>9.4107884478080911E-2</v>
+        <v>9.7217906968953521E-2</v>
       </c>
       <c r="J5">
-        <v>0.28993037238968739</v>
+        <v>0.29761229604335321</v>
       </c>
       <c r="K5">
-        <v>0.53178641148278927</v>
+        <v>0.5325241625239342</v>
       </c>
       <c r="L5">
-        <v>-3.7511295226178507E-2</v>
+        <v>1.529515126914131E-2</v>
       </c>
       <c r="M5">
-        <v>5.5533170709836774</v>
+        <v>7.8754286242893476</v>
       </c>
       <c r="N5">
-        <v>-2.645254148161711E-2</v>
+        <v>-2.6980352711607921E-2</v>
       </c>
       <c r="O5">
-        <v>-3.3352973256136148E-2</v>
+        <v>-3.4017722546166522E-2</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1681,46 +1880,46 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>9.8189487031847447E-2</v>
+        <v>0.112887775898904</v>
       </c>
       <c r="C6">
-        <v>0.30569545283752181</v>
+        <v>0.37228115487312202</v>
       </c>
       <c r="D6">
-        <v>0.1589583774962135</v>
+        <v>0.16019949926865179</v>
       </c>
       <c r="E6">
-        <v>0.63037534121122163</v>
+        <v>0.71445881734510219</v>
       </c>
       <c r="F6">
-        <v>0.8995383435851475</v>
+        <v>1.0255432405840521</v>
       </c>
       <c r="G6">
-        <v>0.53174613885766286</v>
+        <v>0.62009507208127634</v>
       </c>
       <c r="H6">
-        <v>2.328423376866668</v>
+        <v>2.686331151214159</v>
       </c>
       <c r="I6">
-        <v>5.6655259913415072E-2</v>
+        <v>5.6730295575639397E-2</v>
       </c>
       <c r="J6">
-        <v>0.19520251211967601</v>
+        <v>0.19419512529473759</v>
       </c>
       <c r="K6">
-        <v>0.53792945351063648</v>
+        <v>0.53969536423841058</v>
       </c>
       <c r="L6">
-        <v>-0.23058961574691181</v>
+        <v>-0.21796074613732291</v>
       </c>
       <c r="M6">
-        <v>4.4285148583799261</v>
+        <v>4.8923064509303469</v>
       </c>
       <c r="N6">
-        <v>-1.6080996628100201E-2</v>
+        <v>-1.615127020701326E-2</v>
       </c>
       <c r="O6">
-        <v>-2.0265203025056491E-2</v>
+        <v>-2.0368146223158141E-2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1728,46 +1927,46 @@
         <v>19</v>
       </c>
       <c r="B7">
-        <v>0.11963045733543939</v>
+        <v>0.12464625257598</v>
       </c>
       <c r="C7">
-        <v>0.39461841696340222</v>
+        <v>0.4162672989389265</v>
       </c>
       <c r="D7">
-        <v>0.13993453851527021</v>
+        <v>0.13980451931830751</v>
       </c>
       <c r="E7">
-        <v>0.89881828637013816</v>
+        <v>0.93827082524713501</v>
       </c>
       <c r="F7">
-        <v>1.280668801024212</v>
+        <v>1.3461670409336559</v>
       </c>
       <c r="G7">
-        <v>0.75869242516496216</v>
+        <v>0.81453281893399232</v>
       </c>
       <c r="H7">
-        <v>3.9502798271546351</v>
+        <v>4.0288876511128571</v>
       </c>
       <c r="I7">
-        <v>3.739132558752449E-2</v>
+        <v>3.6880800638357837E-2</v>
       </c>
       <c r="J7">
-        <v>0.18352369212686401</v>
+        <v>0.181143189070088</v>
       </c>
       <c r="K7">
-        <v>0.5514006359021203</v>
+        <v>0.55160264900662259</v>
       </c>
       <c r="L7">
-        <v>-0.38412122152833361</v>
+        <v>-0.33478871532815652</v>
       </c>
       <c r="M7">
-        <v>7.0434128921230492</v>
+        <v>7.6222616791966864</v>
       </c>
       <c r="N7">
-        <v>-1.4024738569917389E-2</v>
+        <v>-1.3991362546360679E-2</v>
       </c>
       <c r="O7">
-        <v>-1.7708187032548232E-2</v>
+        <v>-1.7671388558635471E-2</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
@@ -1775,46 +1974,46 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>0.1075952287429762</v>
+        <v>0.11333872861132969</v>
       </c>
       <c r="C8">
-        <v>0.35457862430580089</v>
+        <v>0.37950426466092568</v>
       </c>
       <c r="D8">
-        <v>0.12541497232581461</v>
+        <v>0.12609860710361531</v>
       </c>
       <c r="E8">
-        <v>0.90033754872590932</v>
+        <v>0.93805780376679426</v>
       </c>
       <c r="F8">
-        <v>1.2820746193634149</v>
+        <v>1.341731639283829</v>
       </c>
       <c r="G8">
-        <v>0.75124746283013322</v>
+        <v>0.79564373162553792</v>
       </c>
       <c r="H8">
-        <v>3.8519130956488858</v>
+        <v>3.9449631942002719</v>
       </c>
       <c r="I8">
-        <v>3.7703836472415798E-2</v>
+        <v>3.6252994195740032E-2</v>
       </c>
       <c r="J8">
-        <v>0.16959300826029219</v>
+        <v>0.16657219560625169</v>
       </c>
       <c r="K8">
-        <v>0.55016861946001017</v>
+        <v>0.55041059602649001</v>
       </c>
       <c r="L8">
-        <v>-0.4360733103079843</v>
+        <v>-0.41869964809949622</v>
       </c>
       <c r="M8">
-        <v>6.6458448035494548</v>
+        <v>7.2074308556288189</v>
       </c>
       <c r="N8">
-        <v>-1.256803747629154E-2</v>
+        <v>-1.2616081337978461E-2</v>
       </c>
       <c r="O8">
-        <v>-1.5869292419537731E-2</v>
+        <v>-1.5935331363053688E-2</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
@@ -1822,46 +2021,46 @@
         <v>21</v>
       </c>
       <c r="B9">
-        <v>0.1007472330310666</v>
+        <v>0.1057605666938425</v>
       </c>
       <c r="C9">
-        <v>0.33056138299793281</v>
+        <v>0.3537116137195751</v>
       </c>
       <c r="D9">
-        <v>0.1215818500536487</v>
+        <v>0.1226352721806382</v>
       </c>
       <c r="E9">
-        <v>0.87542262524636516</v>
+        <v>0.90097094843341641</v>
       </c>
       <c r="F9">
-        <v>1.253594743118666</v>
+        <v>1.291167405609279</v>
       </c>
       <c r="G9">
-        <v>0.70072813472383233</v>
+        <v>0.74015883857446785</v>
       </c>
       <c r="H9">
-        <v>3.3230711546008642</v>
+        <v>3.4346361958814442</v>
       </c>
       <c r="I9">
-        <v>4.2706718810726539E-2</v>
+        <v>4.1337476732712271E-2</v>
       </c>
       <c r="J9">
-        <v>0.16893286477627009</v>
+        <v>0.16733665640162279</v>
       </c>
       <c r="K9">
-        <v>0.54480434591670035</v>
+        <v>0.54720529801324502</v>
       </c>
       <c r="L9">
-        <v>-0.41993953543750329</v>
+        <v>-0.43873252398142149</v>
       </c>
       <c r="M9">
-        <v>6.0922987424699571</v>
+        <v>6.573821805371673</v>
       </c>
       <c r="N9">
-        <v>-1.2198039115421401E-2</v>
+        <v>-1.2287296362464079E-2</v>
       </c>
       <c r="O9">
-        <v>-1.5398396106737419E-2</v>
+        <v>-1.551538222011525E-2</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1869,46 +2068,46 @@
         <v>22</v>
       </c>
       <c r="B10">
-        <v>0.1135125131472404</v>
+        <v>0.1204754991568919</v>
       </c>
       <c r="C10">
-        <v>0.37550776664541979</v>
+        <v>0.40787004765432322</v>
       </c>
       <c r="D10">
-        <v>0.13436031385193489</v>
+        <v>0.13725458470392041</v>
       </c>
       <c r="E10">
-        <v>0.88409527996709858</v>
+        <v>0.9117674473232148</v>
       </c>
       <c r="F10">
-        <v>1.2676422113868751</v>
+        <v>1.312904015854085</v>
       </c>
       <c r="G10">
-        <v>0.71611167065412085</v>
+        <v>0.7692194800338743</v>
       </c>
       <c r="H10">
-        <v>3.4438752835739139</v>
+        <v>3.6521929175196872</v>
       </c>
       <c r="I10">
-        <v>4.3434206999395118E-2</v>
+        <v>4.3055740919718317E-2</v>
       </c>
       <c r="J10">
-        <v>0.1807368794066645</v>
+        <v>0.1802318957992893</v>
       </c>
       <c r="K10">
-        <v>0.54642041562000465</v>
+        <v>0.5467417218543047</v>
       </c>
       <c r="L10">
-        <v>-0.36880799675636639</v>
+        <v>-0.35262012880585081</v>
       </c>
       <c r="M10">
-        <v>6.0108427220421481</v>
+        <v>6.8758549766046437</v>
       </c>
       <c r="N10">
-        <v>-1.3471437045841261E-2</v>
+        <v>-1.37436990305924E-2</v>
       </c>
       <c r="O10">
-        <v>-1.7008157120438849E-2</v>
+        <v>-1.7356603995877431E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1918,6 +2117,1534 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>0.13798168658203819</v>
+      </c>
+      <c r="C2">
+        <v>0.45500272483135801</v>
+      </c>
+      <c r="D2">
+        <v>0.1446392354570519</v>
+      </c>
+      <c r="E2">
+        <v>0.86395584910004175</v>
+      </c>
+      <c r="F2">
+        <v>1.2490039899275049</v>
+      </c>
+      <c r="G2">
+        <v>0.69126300652724115</v>
+      </c>
+      <c r="H2">
+        <v>3.931983929041913</v>
+      </c>
+      <c r="I2">
+        <v>3.6291473815293449E-2</v>
+      </c>
+      <c r="J2">
+        <v>0.17852878780819381</v>
+      </c>
+      <c r="K2">
+        <v>0.54966887417218546</v>
+      </c>
+      <c r="L2">
+        <v>-0.21789751899339899</v>
+      </c>
+      <c r="M2">
+        <v>5.3823334700304057</v>
+      </c>
+      <c r="N2">
+        <v>-1.442149111209735E-2</v>
+      </c>
+      <c r="O2">
+        <v>-1.8226436355599031E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>0.19358445218760581</v>
+      </c>
+      <c r="C3">
+        <v>0.61644957895244445</v>
+      </c>
+      <c r="D3">
+        <v>0.22672805903880899</v>
+      </c>
+      <c r="E3">
+        <v>0.83410057162691942</v>
+      </c>
+      <c r="F3">
+        <v>1.219561194297673</v>
+      </c>
+      <c r="G3">
+        <v>0.68474888467422224</v>
+      </c>
+      <c r="H3">
+        <v>2.8401146078392521</v>
+      </c>
+      <c r="I3">
+        <v>6.3823518008448613E-2</v>
+      </c>
+      <c r="J3">
+        <v>0.28196903460949208</v>
+      </c>
+      <c r="K3">
+        <v>0.53377483443708607</v>
+      </c>
+      <c r="L3">
+        <v>-1.818557901398862E-2</v>
+      </c>
+      <c r="M3">
+        <v>4.5947116232853498</v>
+      </c>
+      <c r="N3">
+        <v>-2.2933823706963261E-2</v>
+      </c>
+      <c r="O3">
+        <v>-2.890190799382172E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>9.8621160118798179E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.3168267852013249</v>
+      </c>
+      <c r="D4">
+        <v>0.1174368079993429</v>
+      </c>
+      <c r="E4">
+        <v>0.81263885120483648</v>
+      </c>
+      <c r="F4">
+        <v>1.1749029980677499</v>
+      </c>
+      <c r="G4">
+        <v>0.59641655260090709</v>
+      </c>
+      <c r="H4">
+        <v>2.7943039330582349</v>
+      </c>
+      <c r="I4">
+        <v>3.6076115419194463E-2</v>
+      </c>
+      <c r="J4">
+        <v>0.14723350063482271</v>
+      </c>
+      <c r="K4">
+        <v>0.5437086092715232</v>
+      </c>
+      <c r="L4">
+        <v>-0.39307788872451987</v>
+      </c>
+      <c r="M4">
+        <v>3.3961396599227909</v>
+      </c>
+      <c r="N4">
+        <v>-1.182408966470846E-2</v>
+      </c>
+      <c r="O4">
+        <v>-1.4840604865423769E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>0.20442806805216429</v>
+      </c>
+      <c r="C5">
+        <v>0.66551016315485878</v>
+      </c>
+      <c r="D5">
+        <v>0.27458134927342848</v>
+      </c>
+      <c r="E5">
+        <v>0.83302934534475992</v>
+      </c>
+      <c r="F5">
+        <v>1.190740571014266</v>
+      </c>
+      <c r="G5">
+        <v>0.66897401239796062</v>
+      </c>
+      <c r="H5">
+        <v>2.6450628205902649</v>
+      </c>
+      <c r="I5">
+        <v>8.0375940228167977E-2</v>
+      </c>
+      <c r="J5">
+        <v>0.30257811157529579</v>
+      </c>
+      <c r="K5">
+        <v>0.52913907284768213</v>
+      </c>
+      <c r="L5">
+        <v>6.6262123537941878E-3</v>
+      </c>
+      <c r="M5">
+        <v>4.7087507080558328</v>
+      </c>
+      <c r="N5">
+        <v>-2.737892951397345E-2</v>
+      </c>
+      <c r="O5">
+        <v>-3.4592520943116253E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>0.13145327283179231</v>
+      </c>
+      <c r="C6">
+        <v>0.4100944515981273</v>
+      </c>
+      <c r="D6">
+        <v>0.1564018399906891</v>
+      </c>
+      <c r="E6">
+        <v>0.82779804671766199</v>
+      </c>
+      <c r="F6">
+        <v>1.18802529482451</v>
+      </c>
+      <c r="G6">
+        <v>0.62363935441863705</v>
+      </c>
+      <c r="H6">
+        <v>2.7211011487411949</v>
+      </c>
+      <c r="I6">
+        <v>4.3795290542530618E-2</v>
+      </c>
+      <c r="J6">
+        <v>0.21660585382602829</v>
+      </c>
+      <c r="K6">
+        <v>0.53576158940397356</v>
+      </c>
+      <c r="L6">
+        <v>-0.14974585639159521</v>
+      </c>
+      <c r="M6">
+        <v>3.1740061951981589</v>
+      </c>
+      <c r="N6">
+        <v>-1.577845565614994E-2</v>
+      </c>
+      <c r="O6">
+        <v>-1.9913890625221451E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>0.1251181574217434</v>
+      </c>
+      <c r="C7">
+        <v>0.41286498905573699</v>
+      </c>
+      <c r="D7">
+        <v>0.13357424224511719</v>
+      </c>
+      <c r="E7">
+        <v>0.85703330668029754</v>
+      </c>
+      <c r="F7">
+        <v>1.2175745526100681</v>
+      </c>
+      <c r="G7">
+        <v>0.66450047967216297</v>
+      </c>
+      <c r="H7">
+        <v>3.7635772487033892</v>
+      </c>
+      <c r="I7">
+        <v>3.3253880316057971E-2</v>
+      </c>
+      <c r="J7">
+        <v>0.1655995706532451</v>
+      </c>
+      <c r="K7">
+        <v>0.55099337748344368</v>
+      </c>
+      <c r="L7">
+        <v>-0.25015263743793548</v>
+      </c>
+      <c r="M7">
+        <v>5.1081585180102023</v>
+      </c>
+      <c r="N7">
+        <v>-1.3325994191610929E-2</v>
+      </c>
+      <c r="O7">
+        <v>-1.6841902902398089E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0.1148660276007032</v>
+      </c>
+      <c r="C8">
+        <v>0.38459872847909932</v>
+      </c>
+      <c r="D8">
+        <v>0.1236005335484761</v>
+      </c>
+      <c r="E8">
+        <v>0.92616824529232122</v>
+      </c>
+      <c r="F8">
+        <v>1.2937612172013551</v>
+      </c>
+      <c r="G8">
+        <v>0.7134443804551891</v>
+      </c>
+      <c r="H8">
+        <v>3.8791579503040321</v>
+      </c>
+      <c r="I8">
+        <v>3.0297258143826711E-2</v>
+      </c>
+      <c r="J8">
+        <v>0.15498745812763251</v>
+      </c>
+      <c r="K8">
+        <v>0.55298013245033117</v>
+      </c>
+      <c r="L8">
+        <v>-0.32570821149586759</v>
+      </c>
+      <c r="M8">
+        <v>4.8264916664036024</v>
+      </c>
+      <c r="N8">
+        <v>-1.231452009274211E-2</v>
+      </c>
+      <c r="O8">
+        <v>-1.556364702492833E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>0.11477484206934351</v>
+      </c>
+      <c r="C9">
+        <v>0.37713617864178828</v>
+      </c>
+      <c r="D9">
+        <v>0.1228956838615342</v>
+      </c>
+      <c r="E9">
+        <v>0.92148817651588821</v>
+      </c>
+      <c r="F9">
+        <v>1.294441805189269</v>
+      </c>
+      <c r="G9">
+        <v>0.73664023215245522</v>
+      </c>
+      <c r="H9">
+        <v>3.603891398890477</v>
+      </c>
+      <c r="I9">
+        <v>3.027407769698363E-2</v>
+      </c>
+      <c r="J9">
+        <v>0.1494022666850707</v>
+      </c>
+      <c r="K9">
+        <v>0.55165562913907285</v>
+      </c>
+      <c r="L9">
+        <v>-0.32383581471629058</v>
+      </c>
+      <c r="M9">
+        <v>4.5021342614677993</v>
+      </c>
+      <c r="N9">
+        <v>-1.217520501903332E-2</v>
+      </c>
+      <c r="O9">
+        <v>-1.5372160228678169E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>0.1268039010134917</v>
+      </c>
+      <c r="C10">
+        <v>0.42418691799162977</v>
+      </c>
+      <c r="D10">
+        <v>0.13540809847803559</v>
+      </c>
+      <c r="E10">
+        <v>0.88324591958322674</v>
+      </c>
+      <c r="F10">
+        <v>1.251826199411689</v>
+      </c>
+      <c r="G10">
+        <v>0.7384383200415815</v>
+      </c>
+      <c r="H10">
+        <v>3.614025061409583</v>
+      </c>
+      <c r="I10">
+        <v>3.3894362498591048E-2</v>
+      </c>
+      <c r="J10">
+        <v>0.17076416502265621</v>
+      </c>
+      <c r="K10">
+        <v>0.54966887417218546</v>
+      </c>
+      <c r="L10">
+        <v>-0.27305089032879742</v>
+      </c>
+      <c r="M10">
+        <v>4.4803503819476784</v>
+      </c>
+      <c r="N10">
+        <v>-1.3520470941115709E-2</v>
+      </c>
+      <c r="O10">
+        <v>-1.7077089033369859E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>0.13856003415343879</v>
+      </c>
+      <c r="C2">
+        <v>0.44787035614977871</v>
+      </c>
+      <c r="D2">
+        <v>0.14028932140499331</v>
+      </c>
+      <c r="E2">
+        <v>0.8936212413883815</v>
+      </c>
+      <c r="F2">
+        <v>1.2642501322873041</v>
+      </c>
+      <c r="G2">
+        <v>0.69491997968434249</v>
+      </c>
+      <c r="H2">
+        <v>3.864141558402145</v>
+      </c>
+      <c r="I2">
+        <v>3.4567965935121243E-2</v>
+      </c>
+      <c r="J2">
+        <v>0.1646230236525196</v>
+      </c>
+      <c r="K2">
+        <v>0.55099337748344368</v>
+      </c>
+      <c r="L2">
+        <v>-0.23516635337246861</v>
+      </c>
+      <c r="M2">
+        <v>5.0117150172978251</v>
+      </c>
+      <c r="N2">
+        <v>-1.406028494467822E-2</v>
+      </c>
+      <c r="O2">
+        <v>-1.7737100372331241E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>0.16503906926810691</v>
+      </c>
+      <c r="C3">
+        <v>0.53849178985729496</v>
+      </c>
+      <c r="D3">
+        <v>0.22037222721535471</v>
+      </c>
+      <c r="E3">
+        <v>0.73417221483150774</v>
+      </c>
+      <c r="F3">
+        <v>1.0755353439576349</v>
+      </c>
+      <c r="G3">
+        <v>0.62253659582223375</v>
+      </c>
+      <c r="H3">
+        <v>2.6759121322144099</v>
+      </c>
+      <c r="I3">
+        <v>6.3065630643634518E-2</v>
+      </c>
+      <c r="J3">
+        <v>0.25797886531841269</v>
+      </c>
+      <c r="K3">
+        <v>0.53907284768211916</v>
+      </c>
+      <c r="L3">
+        <v>-6.5960888628154357E-2</v>
+      </c>
+      <c r="M3">
+        <v>4.8171391673625603</v>
+      </c>
+      <c r="N3">
+        <v>-2.2368796849481062E-2</v>
+      </c>
+      <c r="O3">
+        <v>-2.820200396157746E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>9.0193096092591615E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.2873309817786045</v>
+      </c>
+      <c r="D4">
+        <v>0.1123769299311867</v>
+      </c>
+      <c r="E4">
+        <v>0.79781129278080276</v>
+      </c>
+      <c r="F4">
+        <v>1.1227542008885809</v>
+      </c>
+      <c r="G4">
+        <v>0.6350891858590646</v>
+      </c>
+      <c r="H4">
+        <v>2.5735466022403468</v>
+      </c>
+      <c r="I4">
+        <v>3.7637542803677732E-2</v>
+      </c>
+      <c r="J4">
+        <v>0.14838560061057129</v>
+      </c>
+      <c r="K4">
+        <v>0.5437086092715232</v>
+      </c>
+      <c r="L4">
+        <v>-0.42422233017599809</v>
+      </c>
+      <c r="M4">
+        <v>4.0044653506894026</v>
+      </c>
+      <c r="N4">
+        <v>-1.1360199937951379E-2</v>
+      </c>
+      <c r="O4">
+        <v>-1.4284576928616861E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>0.1845934127035439</v>
+      </c>
+      <c r="C5">
+        <v>0.55535986959913719</v>
+      </c>
+      <c r="D5">
+        <v>0.26171712425757448</v>
+      </c>
+      <c r="E5">
+        <v>0.68192148575530576</v>
+      </c>
+      <c r="F5">
+        <v>1.005342325814516</v>
+      </c>
+      <c r="G5">
+        <v>0.62192313497818685</v>
+      </c>
+      <c r="H5">
+        <v>2.1233835473667209</v>
+      </c>
+      <c r="I5">
+        <v>7.9639355038578691E-2</v>
+      </c>
+      <c r="J5">
+        <v>0.29274843971860132</v>
+      </c>
+      <c r="K5">
+        <v>0.5298013245033113</v>
+      </c>
+      <c r="L5">
+        <v>-3.6931924377170633E-2</v>
+      </c>
+      <c r="M5">
+        <v>5.9845119326567309</v>
+      </c>
+      <c r="N5">
+        <v>-2.6418050770276941E-2</v>
+      </c>
+      <c r="O5">
+        <v>-3.3286697143365303E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>0.1066155376261689</v>
+      </c>
+      <c r="C6">
+        <v>0.31034442579281091</v>
+      </c>
+      <c r="D6">
+        <v>0.15630298412958679</v>
+      </c>
+      <c r="E6">
+        <v>0.67629859211648247</v>
+      </c>
+      <c r="F6">
+        <v>0.97366465108319877</v>
+      </c>
+      <c r="G6">
+        <v>0.56827348166864255</v>
+      </c>
+      <c r="H6">
+        <v>2.5732773168663381</v>
+      </c>
+      <c r="I6">
+        <v>4.4705719103907478E-2</v>
+      </c>
+      <c r="J6">
+        <v>0.18830976085874859</v>
+      </c>
+      <c r="K6">
+        <v>0.53907284768211916</v>
+      </c>
+      <c r="L6">
+        <v>-0.21517794606294749</v>
+      </c>
+      <c r="M6">
+        <v>3.7440438287331661</v>
+      </c>
+      <c r="N6">
+        <v>-1.577548340266963E-2</v>
+      </c>
+      <c r="O6">
+        <v>-1.986182432312978E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>0.12381847253330951</v>
+      </c>
+      <c r="C7">
+        <v>0.40793714582382168</v>
+      </c>
+      <c r="D7">
+        <v>0.13079689131842651</v>
+      </c>
+      <c r="E7">
+        <v>0.89049564432098316</v>
+      </c>
+      <c r="F7">
+        <v>1.2497615914643301</v>
+      </c>
+      <c r="G7">
+        <v>0.68112940837558389</v>
+      </c>
+      <c r="H7">
+        <v>3.6764400108383781</v>
+      </c>
+      <c r="I7">
+        <v>3.2478955684443853E-2</v>
+      </c>
+      <c r="J7">
+        <v>0.15929493052988969</v>
+      </c>
+      <c r="K7">
+        <v>0.55165562913907285</v>
+      </c>
+      <c r="L7">
+        <v>-0.26659498447465801</v>
+      </c>
+      <c r="M7">
+        <v>4.8811225662682602</v>
+      </c>
+      <c r="N7">
+        <v>-1.308470959759445E-2</v>
+      </c>
+      <c r="O7">
+        <v>-1.656713252342364E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0.11230730231846919</v>
+      </c>
+      <c r="C8">
+        <v>0.37517608539234981</v>
+      </c>
+      <c r="D8">
+        <v>0.1199556979321065</v>
+      </c>
+      <c r="E8">
+        <v>0.92113946923796575</v>
+      </c>
+      <c r="F8">
+        <v>1.300933967217172</v>
+      </c>
+      <c r="G8">
+        <v>0.73311254399421677</v>
+      </c>
+      <c r="H8">
+        <v>3.8361096970979451</v>
+      </c>
+      <c r="I8">
+        <v>3.0450993588578602E-2</v>
+      </c>
+      <c r="J8">
+        <v>0.14929557271721289</v>
+      </c>
+      <c r="K8">
+        <v>0.54966887417218546</v>
+      </c>
+      <c r="L8">
+        <v>-0.36242497607733509</v>
+      </c>
+      <c r="M8">
+        <v>4.5655813496123674</v>
+      </c>
+      <c r="N8">
+        <v>-1.2003571986275181E-2</v>
+      </c>
+      <c r="O8">
+        <v>-1.5139853414754739E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>0.10708748813944099</v>
+      </c>
+      <c r="C9">
+        <v>0.34529174981386879</v>
+      </c>
+      <c r="D9">
+        <v>0.117414300469124</v>
+      </c>
+      <c r="E9">
+        <v>0.91113534000939489</v>
+      </c>
+      <c r="F9">
+        <v>1.290032737201213</v>
+      </c>
+      <c r="G9">
+        <v>0.72172416424937391</v>
+      </c>
+      <c r="H9">
+        <v>3.365826802096699</v>
+      </c>
+      <c r="I9">
+        <v>3.1962349832441957E-2</v>
+      </c>
+      <c r="J9">
+        <v>0.1485226270840454</v>
+      </c>
+      <c r="K9">
+        <v>0.55033112582781452</v>
+      </c>
+      <c r="L9">
+        <v>-0.36578674154228102</v>
+      </c>
+      <c r="M9">
+        <v>4.4023459503345226</v>
+      </c>
+      <c r="N9">
+        <v>-1.166654661149737E-2</v>
+      </c>
+      <c r="O9">
+        <v>-1.471661471847863E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>0.1187408634670621</v>
+      </c>
+      <c r="C10">
+        <v>0.39555627656068948</v>
+      </c>
+      <c r="D10">
+        <v>0.13377331346502919</v>
+      </c>
+      <c r="E10">
+        <v>0.92202145340473685</v>
+      </c>
+      <c r="F10">
+        <v>1.3192095605404981</v>
+      </c>
+      <c r="G10">
+        <v>0.669897251484318</v>
+      </c>
+      <c r="H10">
+        <v>3.6051394569677639</v>
+      </c>
+      <c r="I10">
+        <v>3.4770981254463373E-2</v>
+      </c>
+      <c r="J10">
+        <v>0.1781825056623336</v>
+      </c>
+      <c r="K10">
+        <v>0.54834437086092713</v>
+      </c>
+      <c r="L10">
+        <v>-0.30828655961582618</v>
+      </c>
+      <c r="M10">
+        <v>4.8292342373512067</v>
+      </c>
+      <c r="N10">
+        <v>-1.3268628044109641E-2</v>
+      </c>
+      <c r="O10">
+        <v>-1.6780360064451039E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>0.13772928485224081</v>
+      </c>
+      <c r="C2">
+        <v>0.44421975147207532</v>
+      </c>
+      <c r="D2">
+        <v>0.14028647658886931</v>
+      </c>
+      <c r="E2">
+        <v>0.88865449697761933</v>
+      </c>
+      <c r="F2">
+        <v>1.2556467042168311</v>
+      </c>
+      <c r="G2">
+        <v>0.69041362096066661</v>
+      </c>
+      <c r="H2">
+        <v>3.8364055396091761</v>
+      </c>
+      <c r="I2">
+        <v>3.4570079480513993E-2</v>
+      </c>
+      <c r="J2">
+        <v>0.16488466690538731</v>
+      </c>
+      <c r="K2">
+        <v>0.55099337748344368</v>
+      </c>
+      <c r="L2">
+        <v>-0.23452324073042871</v>
+      </c>
+      <c r="M2">
+        <v>5.0079516528628041</v>
+      </c>
+      <c r="N2">
+        <v>-1.4059733095499211E-2</v>
+      </c>
+      <c r="O2">
+        <v>-1.7738460384433389E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>0.1606320368676806</v>
+      </c>
+      <c r="C3">
+        <v>0.52222464393575585</v>
+      </c>
+      <c r="D3">
+        <v>0.22046802518784631</v>
+      </c>
+      <c r="E3">
+        <v>0.71739477787432882</v>
+      </c>
+      <c r="F3">
+        <v>1.052690190942845</v>
+      </c>
+      <c r="G3">
+        <v>0.60685808229704297</v>
+      </c>
+      <c r="H3">
+        <v>2.5788839534982069</v>
+      </c>
+      <c r="I3">
+        <v>6.3868541962095168E-2</v>
+      </c>
+      <c r="J3">
+        <v>0.25897988370550101</v>
+      </c>
+      <c r="K3">
+        <v>0.53907284768211916</v>
+      </c>
+      <c r="L3">
+        <v>-6.4562229552376948E-2</v>
+      </c>
+      <c r="M3">
+        <v>4.8129459946379596</v>
+      </c>
+      <c r="N3">
+        <v>-2.2388715327330649E-2</v>
+      </c>
+      <c r="O3">
+        <v>-2.8223521389346719E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>8.8891304422042017E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.28254635122283223</v>
+      </c>
+      <c r="D4">
+        <v>0.11236538479647851</v>
+      </c>
+      <c r="E4">
+        <v>0.78562054932502456</v>
+      </c>
+      <c r="F4">
+        <v>1.1062561905895809</v>
+      </c>
+      <c r="G4">
+        <v>0.62206827933713049</v>
+      </c>
+      <c r="H4">
+        <v>2.5139916275716772</v>
+      </c>
+      <c r="I4">
+        <v>3.7854350648328032E-2</v>
+      </c>
+      <c r="J4">
+        <v>0.1486162233993161</v>
+      </c>
+      <c r="K4">
+        <v>0.54304635761589404</v>
+      </c>
+      <c r="L4">
+        <v>-0.4239608214734471</v>
+      </c>
+      <c r="M4">
+        <v>4.0020401948395969</v>
+      </c>
+      <c r="N4">
+        <v>-1.136736012196664E-2</v>
+      </c>
+      <c r="O4">
+        <v>-1.428789648842534E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5">
+        <v>0.18016893414984969</v>
+      </c>
+      <c r="C5">
+        <v>0.52964794422086137</v>
+      </c>
+      <c r="D5">
+        <v>0.26175201076401661</v>
+      </c>
+      <c r="E5">
+        <v>0.66989493319412219</v>
+      </c>
+      <c r="F5">
+        <v>0.97955221174660312</v>
+      </c>
+      <c r="G5">
+        <v>0.59980006739241709</v>
+      </c>
+      <c r="H5">
+        <v>2.0657726428662611</v>
+      </c>
+      <c r="I5">
+        <v>8.011328735092782E-2</v>
+      </c>
+      <c r="J5">
+        <v>0.29389045711649442</v>
+      </c>
+      <c r="K5">
+        <v>0.52913907284768213</v>
+      </c>
+      <c r="L5">
+        <v>-3.9128518402014048E-2</v>
+      </c>
+      <c r="M5">
+        <v>5.9792174807398606</v>
+      </c>
+      <c r="N5">
+        <v>-2.6431854397644259E-2</v>
+      </c>
+      <c r="O5">
+        <v>-3.3301098077227809E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6">
+        <v>0.10285453967243741</v>
+      </c>
+      <c r="C6">
+        <v>0.29628554951762909</v>
+      </c>
+      <c r="D6">
+        <v>0.156342126166062</v>
+      </c>
+      <c r="E6">
+        <v>0.65193134171348188</v>
+      </c>
+      <c r="F6">
+        <v>0.93902043541252866</v>
+      </c>
+      <c r="G6">
+        <v>0.54786315756670889</v>
+      </c>
+      <c r="H6">
+        <v>2.483365112361037</v>
+      </c>
+      <c r="I6">
+        <v>4.5452285797270661E-2</v>
+      </c>
+      <c r="J6">
+        <v>0.19138489056233321</v>
+      </c>
+      <c r="K6">
+        <v>0.53841059602649</v>
+      </c>
+      <c r="L6">
+        <v>-0.21467251617706279</v>
+      </c>
+      <c r="M6">
+        <v>3.7436379695991442</v>
+      </c>
+      <c r="N6">
+        <v>-1.5794011062665311E-2</v>
+      </c>
+      <c r="O6">
+        <v>-1.9880892861542061E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7">
+        <v>0.12295654761814361</v>
+      </c>
+      <c r="C7">
+        <v>0.40429342346987968</v>
+      </c>
+      <c r="D7">
+        <v>0.1307961685061709</v>
+      </c>
+      <c r="E7">
+        <v>0.88481124227259977</v>
+      </c>
+      <c r="F7">
+        <v>1.2415421243458089</v>
+      </c>
+      <c r="G7">
+        <v>0.67587540873226504</v>
+      </c>
+      <c r="H7">
+        <v>3.6459225801511042</v>
+      </c>
+      <c r="I7">
+        <v>3.2558441465417122E-2</v>
+      </c>
+      <c r="J7">
+        <v>0.1594463558960279</v>
+      </c>
+      <c r="K7">
+        <v>0.55099337748344368</v>
+      </c>
+      <c r="L7">
+        <v>-0.26587847751828619</v>
+      </c>
+      <c r="M7">
+        <v>4.885920987002498</v>
+      </c>
+      <c r="N7">
+        <v>-1.308955546877986E-2</v>
+      </c>
+      <c r="O7">
+        <v>-1.6572329098021719E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>0.1113947711463997</v>
+      </c>
+      <c r="C8">
+        <v>0.37137375783755838</v>
+      </c>
+      <c r="D8">
+        <v>0.11997443845006189</v>
+      </c>
+      <c r="E8">
+        <v>0.9138893883817325</v>
+      </c>
+      <c r="F8">
+        <v>1.292646952070561</v>
+      </c>
+      <c r="G8">
+        <v>0.72497744144504439</v>
+      </c>
+      <c r="H8">
+        <v>3.794411899990191</v>
+      </c>
+      <c r="I8">
+        <v>3.0540278622201981E-2</v>
+      </c>
+      <c r="J8">
+        <v>0.14929557271721261</v>
+      </c>
+      <c r="K8">
+        <v>0.54966887417218546</v>
+      </c>
+      <c r="L8">
+        <v>-0.36196769851530358</v>
+      </c>
+      <c r="M8">
+        <v>4.5703991694973292</v>
+      </c>
+      <c r="N8">
+        <v>-1.2008000985588419E-2</v>
+      </c>
+      <c r="O8">
+        <v>-1.5144466713151899E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>0.1059195957272384</v>
+      </c>
+      <c r="C9">
+        <v>0.34029497764976752</v>
+      </c>
+      <c r="D9">
+        <v>0.1174458190602269</v>
+      </c>
+      <c r="E9">
+        <v>0.89993139405533318</v>
+      </c>
+      <c r="F9">
+        <v>1.2763568869723469</v>
+      </c>
+      <c r="G9">
+        <v>0.71269907963520462</v>
+      </c>
+      <c r="H9">
+        <v>3.290996924613951</v>
+      </c>
+      <c r="I9">
+        <v>3.208310744669704E-2</v>
+      </c>
+      <c r="J9">
+        <v>0.14890025800507289</v>
+      </c>
+      <c r="K9">
+        <v>0.55033112582781452</v>
+      </c>
+      <c r="L9">
+        <v>-0.36500579126014471</v>
+      </c>
+      <c r="M9">
+        <v>4.3993556202331421</v>
+      </c>
+      <c r="N9">
+        <v>-1.167170987077211E-2</v>
+      </c>
+      <c r="O9">
+        <v>-1.4725264335108091E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>0.1174342044890803</v>
+      </c>
+      <c r="C10">
+        <v>0.39003486341876398</v>
+      </c>
+      <c r="D10">
+        <v>0.13379689612795009</v>
+      </c>
+      <c r="E10">
+        <v>0.90958525585391303</v>
+      </c>
+      <c r="F10">
+        <v>1.3034786877995079</v>
+      </c>
+      <c r="G10">
+        <v>0.65740787043197224</v>
+      </c>
+      <c r="H10">
+        <v>3.5471594703125922</v>
+      </c>
+      <c r="I10">
+        <v>3.496392986394567E-2</v>
+      </c>
+      <c r="J10">
+        <v>0.1783318446088292</v>
+      </c>
+      <c r="K10">
+        <v>0.54768211920529808</v>
+      </c>
+      <c r="L10">
+        <v>-0.30730233799431078</v>
+      </c>
+      <c r="M10">
+        <v>4.8275641595910734</v>
+      </c>
+      <c r="N10">
+        <v>-1.327336857059234E-2</v>
+      </c>
+      <c r="O10">
+        <v>-1.6784846316376559E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2">
+        <v>0.1329184211223205</v>
+      </c>
+      <c r="C2">
+        <v>0.42632797967531932</v>
+      </c>
+      <c r="D2">
+        <v>0.17687656088717901</v>
+      </c>
+      <c r="E2">
+        <v>0.79621287953578279</v>
+      </c>
+      <c r="F2">
+        <v>1.1309040896749509</v>
+      </c>
+      <c r="G2">
+        <v>0.63061905511249605</v>
+      </c>
+      <c r="H2">
+        <v>3.6778467917357771</v>
+      </c>
+      <c r="I2">
+        <v>0.23861526912702369</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3">
+        <v>0.1316867894369903</v>
+      </c>
+      <c r="C3">
+        <v>0.3949278570468151</v>
+      </c>
+      <c r="D3">
+        <v>0.17323876572709981</v>
+      </c>
+      <c r="E3">
+        <v>0.7123503941391045</v>
+      </c>
+      <c r="F3">
+        <v>0.9951764590458132</v>
+      </c>
+      <c r="G3">
+        <v>0.48582491290542401</v>
+      </c>
+      <c r="H3">
+        <v>3.285870753970805</v>
+      </c>
+      <c r="I3">
+        <v>0.25425096619230342</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:Q10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1934,52 +3661,52 @@
         <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="L1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="N1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="O1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="P1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -1987,52 +3714,52 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>0.19986373794438819</v>
+        <v>0.20442806805216429</v>
       </c>
       <c r="C2">
-        <v>0.18303007458380149</v>
+        <v>0.1845934127035439</v>
       </c>
       <c r="D2">
-        <v>0.18167671597822849</v>
+        <v>0.18311858651897919</v>
       </c>
       <c r="E2">
-        <v>0.18032335737265551</v>
+        <v>0.18164376033441451</v>
       </c>
       <c r="F2">
-        <v>0.17896999876708239</v>
+        <v>0.18016893414984969</v>
       </c>
       <c r="G2">
-        <v>0.17761664016150941</v>
+        <v>0.17869410796528509</v>
       </c>
       <c r="H2">
-        <v>0.17490992295036331</v>
+        <v>0.1754183358471034</v>
       </c>
       <c r="I2">
-        <v>0.17220320573921721</v>
+        <v>0.17231008745491119</v>
       </c>
       <c r="J2">
-        <v>0.1694964885280712</v>
+        <v>0.16965809591996681</v>
       </c>
       <c r="K2">
-        <v>1.3533586055730069E-3</v>
+        <v>1.474826184564709E-3</v>
       </c>
       <c r="L2">
-        <v>2.706717211146042E-3</v>
+        <v>2.949652369129419E-3</v>
       </c>
       <c r="M2">
-        <v>4.0600758167191331E-3</v>
+        <v>4.4244785536941278E-3</v>
       </c>
       <c r="N2">
-        <v>5.4134344222921127E-3</v>
+        <v>5.8993047382588093E-3</v>
       </c>
       <c r="O2">
-        <v>8.1201516334381829E-3</v>
+        <v>9.1750768564404783E-3</v>
       </c>
       <c r="P2">
-        <v>1.0826868844584279E-2</v>
+        <v>1.228332524863263E-2</v>
       </c>
       <c r="Q2">
-        <v>1.353358605573027E-2</v>
+        <v>1.4935316783577041E-2</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -2040,52 +3767,52 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <v>0.18941950575474251</v>
+        <v>0.19358445218760581</v>
       </c>
       <c r="C3">
-        <v>0.16527151482840949</v>
+        <v>0.16503906926810691</v>
       </c>
       <c r="D3">
-        <v>0.16406912461110401</v>
+        <v>0.1635700584679648</v>
       </c>
       <c r="E3">
-        <v>0.1628667343937984</v>
+        <v>0.16210104766782271</v>
       </c>
       <c r="F3">
-        <v>0.16166434417649281</v>
+        <v>0.1606320368676806</v>
       </c>
       <c r="G3">
-        <v>0.1604619539591873</v>
+        <v>0.15927574749747711</v>
       </c>
       <c r="H3">
-        <v>0.15805717352457621</v>
+        <v>0.15715854778586341</v>
       </c>
       <c r="I3">
-        <v>0.15565239308996501</v>
+        <v>0.1547461759946436</v>
       </c>
       <c r="J3">
-        <v>0.15324761265535389</v>
+        <v>0.15236499740475681</v>
       </c>
       <c r="K3">
-        <v>1.2023902173055321E-3</v>
+        <v>1.469010800142112E-3</v>
       </c>
       <c r="L3">
-        <v>2.4047804346110919E-3</v>
+        <v>2.9380216002842241E-3</v>
       </c>
       <c r="M3">
-        <v>3.607170651916652E-3</v>
+        <v>4.4070324004263361E-3</v>
       </c>
       <c r="N3">
-        <v>4.8095608692221847E-3</v>
+        <v>5.7633217706298534E-3</v>
       </c>
       <c r="O3">
-        <v>7.2143413038333326E-3</v>
+        <v>7.8805214822435243E-3</v>
       </c>
       <c r="P3">
-        <v>9.6191217384444527E-3</v>
+        <v>1.0292893273463281E-2</v>
       </c>
       <c r="Q3">
-        <v>1.2023902173055601E-2</v>
+        <v>1.2674071863350071E-2</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -2093,52 +3820,52 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>0.131077172098511</v>
+        <v>0.13798168658203819</v>
       </c>
       <c r="C4">
-        <v>0.13153948434986731</v>
+        <v>0.13856003415343879</v>
       </c>
       <c r="D4">
-        <v>0.13124834342080399</v>
+        <v>0.13828311771970619</v>
       </c>
       <c r="E4">
-        <v>0.1309572024917407</v>
+        <v>0.13800620128597349</v>
       </c>
       <c r="F4">
-        <v>0.13066606156267749</v>
+        <v>0.13772928485224081</v>
       </c>
       <c r="G4">
-        <v>0.13037492063361419</v>
+        <v>0.13745236841850819</v>
       </c>
       <c r="H4">
-        <v>0.12979263877548769</v>
+        <v>0.13689853555104289</v>
       </c>
       <c r="I4">
-        <v>0.1292103569173611</v>
+        <v>0.1363447026835776</v>
       </c>
       <c r="J4">
-        <v>0.12862807505923449</v>
+        <v>0.1357908698161123</v>
       </c>
       <c r="K4">
-        <v>2.9114092906326611E-4</v>
+        <v>2.7691643373264912E-4</v>
       </c>
       <c r="L4">
-        <v>5.8228185812655986E-4</v>
+        <v>5.5383286746529814E-4</v>
       </c>
       <c r="M4">
-        <v>8.7342278718982591E-4</v>
+        <v>8.3074930119797497E-4</v>
       </c>
       <c r="N4">
-        <v>1.164563716253092E-3</v>
+        <v>1.107665734930652E-3</v>
       </c>
       <c r="O4">
-        <v>1.7468455743796241E-3</v>
+        <v>1.6614986023959499E-3</v>
       </c>
       <c r="P4">
-        <v>2.3291274325061839E-3</v>
+        <v>2.2153314698612481E-3</v>
       </c>
       <c r="Q4">
-        <v>2.9114092906327438E-3</v>
+        <v>2.7691643373265462E-3</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -2146,52 +3873,52 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>0.12102960693777599</v>
+        <v>0.1251181574217434</v>
       </c>
       <c r="C5">
-        <v>0.1205097591770521</v>
+        <v>0.12381847253330951</v>
       </c>
       <c r="D5">
-        <v>0.1202166585631812</v>
+        <v>0.12351674982414509</v>
       </c>
       <c r="E5">
-        <v>0.1199235579493103</v>
+        <v>0.1232348173740095</v>
       </c>
       <c r="F5">
-        <v>0.11963045733543939</v>
+        <v>0.12295654761814361</v>
       </c>
       <c r="G5">
-        <v>0.1193373567215686</v>
+        <v>0.1226782778622776</v>
       </c>
       <c r="H5">
-        <v>0.1187511554938268</v>
+        <v>0.1221217383505457</v>
       </c>
       <c r="I5">
-        <v>0.118164954266085</v>
+        <v>0.1215651988388138</v>
       </c>
       <c r="J5">
-        <v>0.11757875303834329</v>
+        <v>0.1210086593270818</v>
       </c>
       <c r="K5">
-        <v>2.9310061387087532E-4</v>
+        <v>3.017227091644259E-4</v>
       </c>
       <c r="L5">
-        <v>5.8620122774176442E-4</v>
+        <v>5.836551592999506E-4</v>
       </c>
       <c r="M5">
-        <v>8.7930184161263969E-4</v>
+        <v>8.6192491516590142E-4</v>
       </c>
       <c r="N5">
-        <v>1.1724024554835011E-3</v>
+        <v>1.14019467103188E-3</v>
       </c>
       <c r="O5">
-        <v>1.7586036832252789E-3</v>
+        <v>1.696734182763809E-3</v>
       </c>
       <c r="P5">
-        <v>2.3448049109670438E-3</v>
+        <v>2.2532736944957392E-3</v>
       </c>
       <c r="Q5">
-        <v>2.9310061387088078E-3</v>
+        <v>2.8098132062276682E-3</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -2199,52 +3926,52 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>0.118115864066305</v>
+        <v>0.1268039010134917</v>
       </c>
       <c r="C6">
-        <v>0.1148532238115265</v>
+        <v>0.1187408634670621</v>
       </c>
       <c r="D6">
-        <v>0.1144063202567645</v>
+        <v>0.1183053104744015</v>
       </c>
       <c r="E6">
-        <v>0.11395941670200239</v>
+        <v>0.1178697574817409</v>
       </c>
       <c r="F6">
-        <v>0.1135125131472404</v>
+        <v>0.1174342044890803</v>
       </c>
       <c r="G6">
-        <v>0.1130656095924784</v>
+        <v>0.11699865149641971</v>
       </c>
       <c r="H6">
-        <v>0.11217180248295421</v>
+        <v>0.1161275455110985</v>
       </c>
       <c r="I6">
-        <v>0.1112779953734301</v>
+        <v>0.1152564395257773</v>
       </c>
       <c r="J6">
-        <v>0.110384188263906</v>
+        <v>0.1143853335404561</v>
       </c>
       <c r="K6">
-        <v>4.4690355476205418E-4</v>
+        <v>4.3555299266059833E-4</v>
       </c>
       <c r="L6">
-        <v>8.9380710952410847E-4</v>
+        <v>8.711059853211689E-4</v>
       </c>
       <c r="M6">
-        <v>1.340710664286149E-3</v>
+        <v>1.3066589779817811E-3</v>
       </c>
       <c r="N6">
-        <v>1.787614219048189E-3</v>
+        <v>1.7422119706423931E-3</v>
       </c>
       <c r="O6">
-        <v>2.6814213285722981E-3</v>
+        <v>2.61331795596359E-3</v>
       </c>
       <c r="P6">
-        <v>3.5752284380964061E-3</v>
+        <v>3.484423941284787E-3</v>
       </c>
       <c r="Q6">
-        <v>4.4690355476205423E-3</v>
+        <v>4.3555299266059833E-3</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2252,52 +3979,52 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>0.10986625441198231</v>
+        <v>0.1148660276007032</v>
       </c>
       <c r="C7">
-        <v>0.1084888988507679</v>
+        <v>0.11230730231846919</v>
       </c>
       <c r="D7">
-        <v>0.1081910088148373</v>
+        <v>0.1120031252611127</v>
       </c>
       <c r="E7">
-        <v>0.1078931187789068</v>
+        <v>0.1116989482037562</v>
       </c>
       <c r="F7">
-        <v>0.1075952287429762</v>
+        <v>0.1113947711463997</v>
       </c>
       <c r="G7">
-        <v>0.10729733870704571</v>
+        <v>0.1110905940890432</v>
       </c>
       <c r="H7">
-        <v>0.1067015586351845</v>
+        <v>0.1104822399743302</v>
       </c>
       <c r="I7">
-        <v>0.1061057785633234</v>
+        <v>0.1098738858596171</v>
       </c>
       <c r="J7">
-        <v>0.1055099984914623</v>
+        <v>0.1092655317449041</v>
       </c>
       <c r="K7">
-        <v>2.9789003593060082E-4</v>
+        <v>3.0417705735649719E-4</v>
       </c>
       <c r="L7">
-        <v>5.9578007186117388E-4</v>
+        <v>6.083541147129945E-4</v>
       </c>
       <c r="M7">
-        <v>8.936701077917053E-4</v>
+        <v>9.125311720695195E-4</v>
       </c>
       <c r="N7">
-        <v>1.1915601437222641E-3</v>
+        <v>1.2167082294260311E-3</v>
       </c>
       <c r="O7">
-        <v>1.7873402155833969E-3</v>
+        <v>1.825062344139039E-3</v>
       </c>
       <c r="P7">
-        <v>2.383120287444529E-3</v>
+        <v>2.4334164588520608E-3</v>
       </c>
       <c r="Q7">
-        <v>2.9789003593056612E-3</v>
+        <v>3.0417705735650839E-3</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2305,52 +4032,52 @@
         <v>21</v>
       </c>
       <c r="B8">
-        <v>0.1046243249782412</v>
+        <v>0.11477484206934351</v>
       </c>
       <c r="C8">
-        <v>0.10205445913365251</v>
+        <v>0.10708748813944099</v>
       </c>
       <c r="D8">
-        <v>0.1016187170994572</v>
+        <v>0.1066981906687068</v>
       </c>
       <c r="E8">
-        <v>0.1011829750652619</v>
+        <v>0.1063088931979726</v>
       </c>
       <c r="F8">
-        <v>0.1007472330310666</v>
+        <v>0.1059195957272384</v>
       </c>
       <c r="G8">
-        <v>0.1003114909968712</v>
+        <v>0.1055302982565043</v>
       </c>
       <c r="H8">
-        <v>9.9440006928480568E-2</v>
+        <v>0.1047517033150359</v>
       </c>
       <c r="I8">
-        <v>9.8568522860089894E-2</v>
+        <v>0.1039731083735675</v>
       </c>
       <c r="J8">
-        <v>9.769703879169922E-2</v>
+        <v>0.10319451343209909</v>
       </c>
       <c r="K8">
-        <v>4.3574203419530222E-4</v>
+        <v>3.8929747073418453E-4</v>
       </c>
       <c r="L8">
-        <v>8.7148406839065995E-4</v>
+        <v>7.7859494146836905E-4</v>
       </c>
       <c r="M8">
-        <v>1.307226102585976E-3</v>
+        <v>1.167892412202554E-3</v>
       </c>
       <c r="N8">
-        <v>1.742968136781306E-3</v>
+        <v>1.5571898829367381E-3</v>
       </c>
       <c r="O8">
-        <v>2.6144522051719798E-3</v>
+        <v>2.3357848244051349E-3</v>
       </c>
       <c r="P8">
-        <v>3.4859362735626541E-3</v>
+        <v>3.1143797658735178E-3</v>
       </c>
       <c r="Q8">
-        <v>4.3574203419533284E-3</v>
+        <v>3.8929747073419012E-3</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -2358,52 +4085,52 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>0.13434919632155981</v>
+        <v>0.13145327283179231</v>
       </c>
       <c r="C9">
-        <v>0.10158371692667011</v>
+        <v>0.1066155376261689</v>
       </c>
       <c r="D9">
-        <v>0.1004523069617292</v>
+        <v>0.10536187164159171</v>
       </c>
       <c r="E9">
-        <v>9.9320896996788352E-2</v>
+        <v>0.1041082056570146</v>
       </c>
       <c r="F9">
-        <v>9.8189487031847447E-2</v>
+        <v>0.10285453967243741</v>
       </c>
       <c r="G9">
-        <v>9.7058077066906556E-2</v>
+        <v>0.10160087368786019</v>
       </c>
       <c r="H9">
-        <v>9.4795257137024774E-2</v>
+        <v>9.9093541718705921E-2</v>
       </c>
       <c r="I9">
-        <v>9.253243720714302E-2</v>
+        <v>9.6586209749551566E-2</v>
       </c>
       <c r="J9">
-        <v>9.026961727726121E-2</v>
+        <v>9.4078877780397238E-2</v>
       </c>
       <c r="K9">
-        <v>1.131409964940891E-3</v>
+        <v>1.2536659845771849E-3</v>
       </c>
       <c r="L9">
-        <v>2.2628199298817542E-3</v>
+        <v>2.5073319691543421E-3</v>
       </c>
       <c r="M9">
-        <v>3.394229894822659E-3</v>
+        <v>3.760997953731512E-3</v>
       </c>
       <c r="N9">
-        <v>4.52563985976355E-3</v>
+        <v>5.014663938308711E-3</v>
       </c>
       <c r="O9">
-        <v>6.7884597896453319E-3</v>
+        <v>7.5219959074630111E-3</v>
       </c>
       <c r="P9">
-        <v>9.0512797195270861E-3</v>
+        <v>1.002932787661737E-2</v>
       </c>
       <c r="Q9">
-        <v>1.1314099649408899E-2</v>
+        <v>1.2536659845771689E-2</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -2411,52 +4138,52 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>8.6045306736299759E-2</v>
+        <v>9.8621160118798179E-2</v>
       </c>
       <c r="C10">
-        <v>8.4738548852253043E-2</v>
+        <v>9.0193096092591615E-2</v>
       </c>
       <c r="D10">
-        <v>8.4278686885376597E-2</v>
+        <v>8.9759165535741731E-2</v>
       </c>
       <c r="E10">
-        <v>8.3818824918500193E-2</v>
+        <v>8.9325234978891901E-2</v>
       </c>
       <c r="F10">
-        <v>8.3358962951623747E-2</v>
+        <v>8.8891304422042017E-2</v>
       </c>
       <c r="G10">
-        <v>8.2899100984747329E-2</v>
+        <v>8.8457373865192188E-2</v>
       </c>
       <c r="H10">
-        <v>8.1979377050994465E-2</v>
+        <v>8.7589512751492446E-2</v>
       </c>
       <c r="I10">
-        <v>8.1059653117241601E-2</v>
+        <v>8.6721651637792718E-2</v>
       </c>
       <c r="J10">
-        <v>8.0139929183488778E-2</v>
+        <v>8.5853790524093004E-2</v>
       </c>
       <c r="K10">
-        <v>4.5986196687644593E-4</v>
+        <v>4.3393055684988469E-4</v>
       </c>
       <c r="L10">
-        <v>9.1972393375285011E-4</v>
+        <v>8.6786111369971386E-4</v>
       </c>
       <c r="M10">
-        <v>1.379585900629296E-3</v>
+        <v>1.301791670549599E-3</v>
       </c>
       <c r="N10">
-        <v>1.8394478675057141E-3</v>
+        <v>1.7357222273994279E-3</v>
       </c>
       <c r="O10">
-        <v>2.7591718012585781E-3</v>
+        <v>2.6035833410991689E-3</v>
       </c>
       <c r="P10">
-        <v>3.6788957350114421E-3</v>
+        <v>3.4714444547988971E-3</v>
       </c>
       <c r="Q10">
-        <v>4.5986196687642644E-3</v>
+        <v>4.3393055684986109E-3</v>
       </c>
     </row>
   </sheetData>
@@ -2464,8 +4191,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:Q10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -2474,52 +4201,52 @@
         <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="L1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="O1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="P1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="Q1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -2527,52 +4254,52 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>0.70509485683100503</v>
+        <v>0.66551016315485878</v>
       </c>
       <c r="C2">
-        <v>0.63559160557845107</v>
+        <v>0.55535986959913719</v>
       </c>
       <c r="D2">
-        <v>0.62945689622881418</v>
+        <v>0.54674741847004493</v>
       </c>
       <c r="E2">
-        <v>6.134709349636891E-3</v>
+        <v>8.6124511290922579E-3</v>
       </c>
       <c r="F2">
-        <v>0.62334512259638974</v>
+        <v>0.53817683514840609</v>
       </c>
       <c r="G2">
-        <v>1.2246482982061321E-2</v>
+        <v>1.7183034450731108E-2</v>
       </c>
       <c r="H2">
-        <v>0.61725620077977095</v>
+        <v>0.52964794422086137</v>
       </c>
       <c r="I2">
-        <v>1.8335404798680122E-2</v>
+        <v>2.571192537827582E-2</v>
       </c>
       <c r="J2">
-        <v>0.61119004716901881</v>
+        <v>0.5211605708901309</v>
       </c>
       <c r="K2">
-        <v>2.4401558409432259E-2</v>
+        <v>3.4199298709006287E-2</v>
       </c>
       <c r="L2">
-        <v>0.59912571157712935</v>
+        <v>0.50430968089998707</v>
       </c>
       <c r="M2">
-        <v>3.6465894001321719E-2</v>
+        <v>5.1050188699150123E-2</v>
       </c>
       <c r="N2">
-        <v>0.58715145273531166</v>
+        <v>0.48899136889446948</v>
       </c>
       <c r="O2">
-        <v>4.8440152843139413E-2</v>
+        <v>6.636850070466771E-2</v>
       </c>
       <c r="P2">
-        <v>0.57526661216240382</v>
+        <v>0.47644553210255652</v>
       </c>
       <c r="Q2">
-        <v>6.0324993416047253E-2</v>
+        <v>7.8914337496580722E-2</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -2580,52 +4307,52 @@
         <v>15</v>
       </c>
       <c r="B3">
-        <v>0.67502490657370995</v>
+        <v>0.61644957895244445</v>
       </c>
       <c r="C3">
-        <v>0.56655798033003846</v>
+        <v>0.53849178985729496</v>
       </c>
       <c r="D3">
-        <v>0.56117681685317233</v>
+        <v>0.53277497010086938</v>
       </c>
       <c r="E3">
-        <v>5.3811634768661243E-3</v>
+        <v>5.7168197564255729E-3</v>
       </c>
       <c r="F3">
-        <v>0.55581314810072213</v>
+        <v>0.52749188387653723</v>
       </c>
       <c r="G3">
-        <v>1.0744832229316331E-2</v>
+        <v>1.0999905980757729E-2</v>
       </c>
       <c r="H3">
-        <v>0.55046692084529936</v>
+        <v>0.52222464393575585</v>
       </c>
       <c r="I3">
-        <v>1.6091059484739101E-2</v>
+        <v>1.6267145921539109E-2</v>
       </c>
       <c r="J3">
-        <v>0.54513808200875291</v>
+        <v>0.5161315654615457</v>
       </c>
       <c r="K3">
-        <v>2.141989832128555E-2</v>
+        <v>2.2360224395749251E-2</v>
       </c>
       <c r="L3">
-        <v>0.53453235802360166</v>
+        <v>0.50486678484936232</v>
       </c>
       <c r="M3">
-        <v>3.2025622306436803E-2</v>
+        <v>3.362500500793264E-2</v>
       </c>
       <c r="N3">
-        <v>0.52399555449046264</v>
+        <v>0.49384926793735168</v>
       </c>
       <c r="O3">
-        <v>4.2562425839575813E-2</v>
+        <v>4.4642521919943223E-2</v>
       </c>
       <c r="P3">
-        <v>0.51352725211822092</v>
+        <v>0.48274167093813192</v>
       </c>
       <c r="Q3">
-        <v>5.3030728211817528E-2</v>
+        <v>5.5750118919163039E-2</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -2633,52 +4360,52 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>0.43493137445058588</v>
+        <v>0.45500272483135801</v>
       </c>
       <c r="C4">
-        <v>0.43808458186343813</v>
+        <v>0.44787035614977871</v>
       </c>
       <c r="D4">
-        <v>0.43683088177464091</v>
+        <v>0.44663057233973508</v>
       </c>
       <c r="E4">
-        <v>1.253700088797161E-3</v>
+        <v>1.239783810043527E-3</v>
       </c>
       <c r="F4">
-        <v>0.43557790076077579</v>
+        <v>0.4454141174912738</v>
       </c>
       <c r="G4">
-        <v>2.5066811026622782E-3</v>
+        <v>2.4562386585048608E-3</v>
       </c>
       <c r="H4">
-        <v>0.4343256384880686</v>
+        <v>0.44421975147207532</v>
       </c>
       <c r="I4">
-        <v>3.7589433753694719E-3</v>
+        <v>3.6506046777033951E-3</v>
       </c>
       <c r="J4">
-        <v>0.43307409462287549</v>
+        <v>0.44302599327469361</v>
       </c>
       <c r="K4">
-        <v>5.0104872405625778E-3</v>
+        <v>4.8443628750850509E-3</v>
       </c>
       <c r="L4">
-        <v>0.43057316078111652</v>
+        <v>0.44064029937243138</v>
       </c>
       <c r="M4">
-        <v>7.5114210823215566E-3</v>
+        <v>7.2300567773472268E-3</v>
       </c>
       <c r="N4">
-        <v>0.42807509656898679</v>
+        <v>0.4382570338393712</v>
       </c>
       <c r="O4">
-        <v>1.000948529445128E-2</v>
+        <v>9.6133223104074572E-3</v>
       </c>
       <c r="P4">
-        <v>0.42557989932208118</v>
+        <v>0.43587619473168232</v>
       </c>
       <c r="Q4">
-        <v>1.2504682541356889E-2</v>
+        <v>1.1994161418096391E-2</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -2686,52 +4413,52 @@
         <v>19</v>
       </c>
       <c r="B5">
-        <v>0.39823276722133849</v>
+        <v>0.41286498905573699</v>
       </c>
       <c r="C5">
-        <v>0.3982975934081035</v>
+        <v>0.40793714582382168</v>
       </c>
       <c r="D5">
-        <v>0.39707048855449267</v>
+        <v>0.40672189100770861</v>
       </c>
       <c r="E5">
-        <v>1.227104853610828E-3</v>
+        <v>1.215254816113065E-3</v>
       </c>
       <c r="F5">
-        <v>0.39584409651811592</v>
+        <v>0.40550731699070841</v>
       </c>
       <c r="G5">
-        <v>2.4534968899875831E-3</v>
+        <v>2.4298288331132678E-3</v>
       </c>
       <c r="H5">
-        <v>0.39461841696340222</v>
+        <v>0.40429342346987968</v>
       </c>
       <c r="I5">
-        <v>3.679176444701338E-3</v>
+        <v>3.6437223539419472E-3</v>
       </c>
       <c r="J5">
-        <v>0.39339344955491318</v>
+        <v>0.40308021014238671</v>
       </c>
       <c r="K5">
-        <v>4.9041438531903236E-3</v>
+        <v>4.8569356814349707E-3</v>
       </c>
       <c r="L5">
-        <v>0.39094564983552949</v>
+        <v>0.40065582285663809</v>
       </c>
       <c r="M5">
-        <v>7.3519435725740157E-3</v>
+        <v>7.2813229671835336E-3</v>
       </c>
       <c r="N5">
-        <v>0.38850069467915571</v>
+        <v>0.39823415271306511</v>
       </c>
       <c r="O5">
-        <v>9.7968987289478449E-3</v>
+        <v>9.7029931107566192E-3</v>
       </c>
       <c r="P5">
-        <v>0.38605858140712901</v>
+        <v>0.39581519729305292</v>
       </c>
       <c r="Q5">
-        <v>1.2239012000974551E-2</v>
+        <v>1.2121948530768759E-2</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -2739,52 +4466,52 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>0.39510725866186708</v>
+        <v>0.42418691799162977</v>
       </c>
       <c r="C6">
-        <v>0.38105005421365828</v>
+        <v>0.39555627656068948</v>
       </c>
       <c r="D6">
-        <v>0.3792005814272022</v>
+        <v>0.3937138239246164</v>
       </c>
       <c r="E6">
-        <v>1.8494727864561411E-3</v>
+        <v>1.842452636073078E-3</v>
       </c>
       <c r="F6">
-        <v>0.37735315288332832</v>
+        <v>0.39187335347637631</v>
       </c>
       <c r="G6">
-        <v>3.6969013303300162E-3</v>
+        <v>3.6829230843131722E-3</v>
       </c>
       <c r="H6">
-        <v>0.37550776664541979</v>
+        <v>0.39003486341876398</v>
       </c>
       <c r="I6">
-        <v>5.5422875682384909E-3</v>
+        <v>5.5214131419254464E-3</v>
       </c>
       <c r="J6">
-        <v>0.37366442077845091</v>
+        <v>0.38819835195596519</v>
       </c>
       <c r="K6">
-        <v>7.3856334352074837E-3</v>
+        <v>7.3579246047242863E-3</v>
       </c>
       <c r="L6">
-        <v>0.36998384242517363</v>
+        <v>0.38453125763847812</v>
       </c>
       <c r="M6">
-        <v>1.1066211788484709E-2</v>
+        <v>1.1025018922211419E-2</v>
       </c>
       <c r="N6">
-        <v>0.36631140237506482</v>
+        <v>0.38087205618508801</v>
       </c>
       <c r="O6">
-        <v>1.473865183859357E-2</v>
+        <v>1.4684220375601459E-2</v>
       </c>
       <c r="P6">
-        <v>0.36264708520508132</v>
+        <v>0.37722073327909</v>
       </c>
       <c r="Q6">
-        <v>1.8402969008577019E-2</v>
+        <v>1.8335543281599479E-2</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -2792,52 +4519,52 @@
         <v>20</v>
       </c>
       <c r="B7">
-        <v>0.36240436332752851</v>
+        <v>0.38459872847909932</v>
       </c>
       <c r="C7">
-        <v>0.35820709601322298</v>
+        <v>0.37517608539234981</v>
       </c>
       <c r="D7">
-        <v>0.35699688309538302</v>
+        <v>0.3739078426532868</v>
       </c>
       <c r="E7">
-        <v>1.210212917839959E-3</v>
+        <v>1.268242739063008E-3</v>
       </c>
       <c r="F7">
-        <v>0.35578739264250669</v>
+        <v>0.37264040026952411</v>
       </c>
       <c r="G7">
-        <v>2.4197033707162858E-3</v>
+        <v>2.5356851228257589E-3</v>
       </c>
       <c r="H7">
-        <v>0.35457862430580089</v>
+        <v>0.37137375783755838</v>
       </c>
       <c r="I7">
-        <v>3.6284717074220318E-3</v>
+        <v>3.8023275547913742E-3</v>
       </c>
       <c r="J7">
-        <v>0.35337057773661251</v>
+        <v>0.37010791495405138</v>
       </c>
       <c r="K7">
-        <v>4.8365182766104686E-3</v>
+        <v>5.0681704382984361E-3</v>
       </c>
       <c r="L7">
-        <v>0.35095664850689001</v>
+        <v>0.36757862621991932</v>
       </c>
       <c r="M7">
-        <v>7.2504475063330243E-3</v>
+        <v>7.5974591724304874E-3</v>
       </c>
       <c r="N7">
-        <v>0.3485456021669715</v>
+        <v>0.36505253084382278</v>
       </c>
       <c r="O7">
-        <v>9.6614938462514788E-3</v>
+        <v>1.0123554548526981E-2</v>
       </c>
       <c r="P7">
-        <v>0.34613743593276958</v>
+        <v>0.36252962560516888</v>
       </c>
       <c r="Q7">
-        <v>1.206966008045335E-2</v>
+        <v>1.264645978718093E-2</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -2845,52 +4572,52 @@
         <v>21</v>
       </c>
       <c r="B8">
-        <v>0.34701722256327477</v>
+        <v>0.37713617864178828</v>
       </c>
       <c r="C8">
-        <v>0.33579881525509653</v>
+        <v>0.34529174981386879</v>
       </c>
       <c r="D8">
-        <v>0.3340511230569076</v>
+        <v>0.3436245061555232</v>
       </c>
       <c r="E8">
-        <v>1.7476921981888769E-3</v>
+        <v>1.667243658345585E-3</v>
       </c>
       <c r="F8">
-        <v>0.3323053128862592</v>
+        <v>0.34195891589208749</v>
       </c>
       <c r="G8">
-        <v>3.4935023688372762E-3</v>
+        <v>3.332833921781297E-3</v>
       </c>
       <c r="H8">
-        <v>0.33056138299793281</v>
+        <v>0.34029497764976752</v>
       </c>
       <c r="I8">
-        <v>5.2374322571637211E-3</v>
+        <v>4.9967721641013263E-3</v>
       </c>
       <c r="J8">
-        <v>0.3288193316481246</v>
+        <v>0.33863269005574492</v>
       </c>
       <c r="K8">
-        <v>6.9794836069718702E-3</v>
+        <v>6.6590597581238642E-3</v>
       </c>
       <c r="L8">
-        <v>0.32534085759591141</v>
+        <v>0.33531306132614103</v>
       </c>
       <c r="M8">
-        <v>1.0457957659185059E-2</v>
+        <v>9.9786884877277604E-3</v>
       </c>
       <c r="N8">
-        <v>0.3218698768074239</v>
+        <v>0.33200001874008278</v>
       </c>
       <c r="O8">
-        <v>1.3928938447672569E-2</v>
+        <v>1.329173107378601E-2</v>
       </c>
       <c r="P8">
-        <v>0.31840637538301869</v>
+        <v>0.32869355134986661</v>
       </c>
       <c r="Q8">
-        <v>1.7392439872077729E-2</v>
+        <v>1.6598198464002231E-2</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -2898,52 +4625,52 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>0.46772470388705267</v>
+        <v>0.4100944515981273</v>
       </c>
       <c r="C9">
-        <v>0.31900229526927992</v>
+        <v>0.31034442579281091</v>
       </c>
       <c r="D9">
-        <v>0.31455275631921947</v>
+        <v>0.30564307707199972</v>
       </c>
       <c r="E9">
-        <v>4.4495389500604499E-3</v>
+        <v>4.7013487208111826E-3</v>
       </c>
       <c r="F9">
-        <v>0.31011715561269743</v>
+        <v>0.30095679921631918</v>
       </c>
       <c r="G9">
-        <v>8.8851396565824969E-3</v>
+        <v>9.3876265764916145E-3</v>
       </c>
       <c r="H9">
-        <v>0.30569545283752181</v>
+        <v>0.29628554951762909</v>
       </c>
       <c r="I9">
-        <v>1.3306842431758109E-2</v>
+        <v>1.4058876275181761E-2</v>
       </c>
       <c r="J9">
-        <v>0.30128760778824998</v>
+        <v>0.2916292853735577</v>
       </c>
       <c r="K9">
-        <v>1.7714687481029889E-2</v>
+        <v>1.8715140419253151E-2</v>
       </c>
       <c r="L9">
-        <v>0.29251333057786078</v>
+        <v>0.28236154386715151</v>
       </c>
       <c r="M9">
-        <v>2.6488964691419151E-2</v>
+        <v>2.7982881925659338E-2</v>
       </c>
       <c r="N9">
-        <v>0.28379400446327069</v>
+        <v>0.27315323598457392</v>
       </c>
       <c r="O9">
-        <v>3.5208290806009179E-2</v>
+        <v>3.7191189808236991E-2</v>
       </c>
       <c r="P9">
-        <v>0.27512931161789711</v>
+        <v>0.26400402469096962</v>
       </c>
       <c r="Q9">
-        <v>4.3872983651382813E-2</v>
+        <v>4.6340401101841233E-2</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
@@ -2951,172 +4678,52 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>0.27348499770369988</v>
+        <v>0.3168267852013249</v>
       </c>
       <c r="C10">
-        <v>0.26924640435365571</v>
+        <v>0.2873309817786045</v>
       </c>
       <c r="D10">
-        <v>0.26749344664209967</v>
+        <v>0.2857964755536091</v>
       </c>
       <c r="E10">
-        <v>1.75295771155598E-3</v>
+        <v>1.534506224995402E-3</v>
       </c>
       <c r="F10">
-        <v>0.2657425101806698</v>
+        <v>0.28422916955209082</v>
       </c>
       <c r="G10">
-        <v>3.5038941729859112E-3</v>
+        <v>3.1018122265137338E-3</v>
       </c>
       <c r="H10">
-        <v>0.26399359295411567</v>
+        <v>0.28254635122283223</v>
       </c>
       <c r="I10">
-        <v>5.2528113995400361E-3</v>
+        <v>4.7846305557722726E-3</v>
       </c>
       <c r="J10">
-        <v>0.26224669294894482</v>
+        <v>0.28086530127839943</v>
       </c>
       <c r="K10">
-        <v>6.999711404710951E-3</v>
+        <v>6.4656805002051287E-3</v>
       </c>
       <c r="L10">
-        <v>0.2587589365575455</v>
+        <v>0.27750850040514657</v>
       </c>
       <c r="M10">
-        <v>1.0487467796110209E-2</v>
+        <v>9.8224813734578698E-3</v>
       </c>
       <c r="N10">
-        <v>0.25527922493358779</v>
+        <v>0.27415875466579442</v>
       </c>
       <c r="O10">
-        <v>1.3967179420067919E-2</v>
+        <v>1.3172227112810081E-2</v>
       </c>
       <c r="P10">
-        <v>0.25180754203219302</v>
+        <v>0.27081605181171148</v>
       </c>
       <c r="Q10">
-        <v>1.7438862321462741E-2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>2.37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>2.0699999999999998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>1.93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0.56000000000000005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0.54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0.26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>0.25</v>
+        <v>1.651492996689297E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>